<commit_message>
refactor(core): standardize on single Day 10 candling stage and strict 2-class vision model
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -593,6 +593,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
@@ -633,6 +634,8 @@
         <v/>
       </c>
     </row>
+    <row r="6"/>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
@@ -804,6 +807,8 @@
         <v/>
       </c>
     </row>
+    <row r="15"/>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -835,7 +840,7 @@
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>4. Strict Architectural Tenets: Zero Firebase (100% FastAPI+PostgreSQL), offline SQLite WAL at edge, 3 biological classes, FU branding (#800000).</t>
+          <t>4. Strict Architectural Tenets: Zero Firebase (100% FastAPI+PostgreSQL), offline SQLite WAL at edge, strict 2 biological classes (Fertile, Infertile), Day 10 candling, FU branding (#800000).</t>
         </is>
       </c>
     </row>
@@ -862,7 +867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J117"/>
+  <dimension ref="A1:J116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -877,6 +882,8 @@
     <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
@@ -1784,7 +1791,7 @@
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>Hatch yield forecast calculation based on Day 10 and Day 18 viability rates</t>
+          <t>Hatch yield forecast calculation based on Day 10 fertility viability rate</t>
         </is>
       </c>
       <c r="F20" s="14" t="inlineStr">
@@ -1888,7 +1895,7 @@
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>Advance batch milestone: Day 10 -&gt; Day 18 -&gt; Day 25</t>
+          <t>Advance batch milestone: SETTING -&gt; DAY_10 -&gt; HATCHED -&gt; COMPLETED</t>
         </is>
       </c>
       <c r="F22" s="14" t="inlineStr">
@@ -2096,7 +2103,7 @@
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>Automated background cron to flag batches reaching Day 10, 18, 25</t>
+          <t>Automated background cron to flag batches reaching Day 10 candling milestone</t>
         </is>
       </c>
       <c r="F26" s="14" t="inlineStr">
@@ -2252,7 +2259,7 @@
       </c>
       <c r="E29" s="17" t="inlineStr">
         <is>
-          <t>Get session progress: total eggs candled, fertile, infertile, abnormal counts</t>
+          <t>Get session progress: total eggs candled, fertile, infertile counts</t>
         </is>
       </c>
       <c r="F29" s="17" t="inlineStr">
@@ -2720,7 +2727,7 @@
       </c>
       <c r="E38" s="14" t="inlineStr">
         <is>
-          <t>Longitudinal mortality tracking across batches and candling stages</t>
+          <t>Longitudinal fertility and cull tracking across historical batches</t>
         </is>
       </c>
       <c r="F38" s="14" t="inlineStr">
@@ -2772,7 +2779,7 @@
       </c>
       <c r="E39" s="17" t="inlineStr">
         <is>
-          <t>Progressive loss analysis from Day 10 to Day 18 to Day 25</t>
+          <t>Loss analysis and commercial Penoy recovery on Day 10</t>
         </is>
       </c>
       <c r="F39" s="17" t="inlineStr">
@@ -4384,7 +4391,7 @@
       </c>
       <c r="E70" s="14" t="inlineStr">
         <is>
-          <t>Live counters for Fertile, Infertile, Abnormal, and Manual Review count</t>
+          <t>Live counters for Fertile, Infertile, and Manual Review count</t>
         </is>
       </c>
       <c r="F70" s="14" t="inlineStr">
@@ -4644,7 +4651,7 @@
       </c>
       <c r="E75" s="17" t="inlineStr">
         <is>
-          <t>Table of all batches, stage advancement modal (Day 10/18/25), hatch closure</t>
+          <t>Table of all batches, stage advancement modal (Day 10, Hatched, Completed), hatch closure</t>
         </is>
       </c>
       <c r="F75" s="17" t="inlineStr">
@@ -5263,12 +5270,12 @@
       </c>
       <c r="D87" s="17" t="inlineStr">
         <is>
-          <t>Stage Filter: Day 10, Day 18, Day 25</t>
+          <t>Stage Filter: Setting, Day 10, Hatched, Completed</t>
         </is>
       </c>
       <c r="E87" s="17" t="inlineStr">
         <is>
-          <t>Toggle to filter analysis by candling milestone checkpoint</t>
+          <t>Toggle to filter analysis by incubation stage milestone</t>
         </is>
       </c>
       <c r="F87" s="17" t="inlineStr">
@@ -5593,9 +5600,9 @@
           <t>Codex</t>
         </is>
       </c>
-      <c r="H93" s="18" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="H93" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I93" s="16" t="inlineStr">
@@ -5605,7 +5612,7 @@
       </c>
       <c r="J93" s="17" t="inlineStr">
         <is>
-          <t>Serial loopback test</t>
+          <t>esp32_actuator.ino review</t>
         </is>
       </c>
     </row>
@@ -5679,12 +5686,12 @@
       </c>
       <c r="D95" s="17" t="inlineStr">
         <is>
-          <t>Servo Gate 1 (Fertile Release)</t>
+          <t>Servo Diverter (Fertile Pass-Through)</t>
         </is>
       </c>
       <c r="E95" s="17" t="inlineStr">
         <is>
-          <t>Actuate servo diverter for Fertile eggs into cushioned incubation tray</t>
+          <t>Maintain idle servo position (0 deg) allowing Fertile eggs to continue to incubation tray</t>
         </is>
       </c>
       <c r="F95" s="17" t="inlineStr">
@@ -5731,12 +5738,12 @@
       </c>
       <c r="D96" s="14" t="inlineStr">
         <is>
-          <t>Servo Gate 2 (Infertile / Penoy Salvage)</t>
+          <t>Servo Diverter (Infertile / Penoy Salvage)</t>
         </is>
       </c>
       <c r="E96" s="14" t="inlineStr">
         <is>
-          <t>Actuate servo diverter for Day 10 Penoy salvage sale (@ P14.00)</t>
+          <t>Actuate servo diverter (60 deg) for Day 10 Penoy salvage sale (@ P14.00)</t>
         </is>
       </c>
       <c r="F96" s="14" t="inlineStr">
@@ -5749,9 +5756,9 @@
           <t>Codex</t>
         </is>
       </c>
-      <c r="H96" s="18" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="H96" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I96" s="13" t="inlineStr">
@@ -5761,14 +5768,14 @@
       </c>
       <c r="J96" s="14" t="inlineStr">
         <is>
-          <t>Firmware bench test</t>
+          <t>esp32_actuator.ino review</t>
         </is>
       </c>
     </row>
     <row r="97" ht="22" customHeight="1">
       <c r="A97" s="16" t="inlineStr">
         <is>
-          <t>TASK-FW-SRV-03</t>
+          <t>TASK-FW-KIN-01</t>
         </is>
       </c>
       <c r="B97" s="16" t="inlineStr">
@@ -5783,17 +5790,17 @@
       </c>
       <c r="D97" s="17" t="inlineStr">
         <is>
-          <t>Servo Gate 3 (Abnormal Discard)</t>
+          <t>Kinematic Actuation Delay Timer</t>
         </is>
       </c>
       <c r="E97" s="17" t="inlineStr">
         <is>
-          <t>Actuate servo diverter to cull dead/bursting embryos to waste bin</t>
+          <t>Calculate Delta-t = D / v = 25cm / 12.5cm/s = 2000ms delay before servo firing</t>
         </is>
       </c>
       <c r="F97" s="17" t="inlineStr">
         <is>
-          <t>System Flowchart Node 20</t>
+          <t>Methodology 3.4</t>
         </is>
       </c>
       <c r="G97" s="16" t="inlineStr">
@@ -5801,9 +5808,9 @@
           <t>Codex</t>
         </is>
       </c>
-      <c r="H97" s="18" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="H97" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I97" s="16" t="inlineStr">
@@ -5813,39 +5820,39 @@
       </c>
       <c r="J97" s="17" t="inlineStr">
         <is>
-          <t>Firmware bench test</t>
+          <t>esp32_actuator.ino review</t>
         </is>
       </c>
     </row>
     <row r="98" ht="22" customHeight="1">
       <c r="A98" s="13" t="inlineStr">
         <is>
-          <t>TASK-FW-KIN-01</t>
+          <t>TASK-AI-DS-01</t>
         </is>
       </c>
       <c r="B98" s="13" t="inlineStr">
         <is>
-          <t>Phase 4A: Firmware</t>
+          <t>Phase 2: Dataset</t>
         </is>
       </c>
       <c r="C98" s="14" t="inlineStr">
         <is>
-          <t>Firmware</t>
+          <t>AI &amp; Data</t>
         </is>
       </c>
       <c r="D98" s="14" t="inlineStr">
         <is>
-          <t>Kinematic Actuation Delay Timer</t>
+          <t>Dataset 70/15/15 Stratification Pipeline</t>
         </is>
       </c>
       <c r="E98" s="14" t="inlineStr">
         <is>
-          <t>Calculate Delta-t = D / v = 25cm / 12.5cm/s = 2000ms delay before servo firing</t>
+          <t>Partition 3,000+ candling images into 70% Train, 15% Val, 15% Test across Day 10 candling captures</t>
         </is>
       </c>
       <c r="F98" s="14" t="inlineStr">
         <is>
-          <t>Methodology 3.4</t>
+          <t>IPO Matrix / Meth</t>
         </is>
       </c>
       <c r="G98" s="13" t="inlineStr">
@@ -5853,9 +5860,9 @@
           <t>Codex</t>
         </is>
       </c>
-      <c r="H98" s="15" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="H98" s="18" t="inlineStr">
+        <is>
+          <t>Backlog</t>
         </is>
       </c>
       <c r="I98" s="13" t="inlineStr">
@@ -5865,14 +5872,14 @@
       </c>
       <c r="J98" s="14" t="inlineStr">
         <is>
-          <t>esp32_actuator.ino review</t>
+          <t>test_dataset_stratification.py</t>
         </is>
       </c>
     </row>
     <row r="99" ht="22" customHeight="1">
       <c r="A99" s="16" t="inlineStr">
         <is>
-          <t>TASK-AI-DS-01</t>
+          <t>TASK-AI-DS-02</t>
         </is>
       </c>
       <c r="B99" s="16" t="inlineStr">
@@ -5887,17 +5894,17 @@
       </c>
       <c r="D99" s="17" t="inlineStr">
         <is>
-          <t>Dataset 70/15/15 Stratification Pipeline</t>
+          <t>Whole-Egg YOLO Bounding Box Validator</t>
         </is>
       </c>
       <c r="E99" s="17" t="inlineStr">
         <is>
-          <t>Partition 3,000+ candling images into 70% Train, 15% Val, 15% Test</t>
+          <t>Verify YOLO darknet format [class_id, x, y, w, h] enclosing whole egg</t>
         </is>
       </c>
       <c r="F99" s="17" t="inlineStr">
         <is>
-          <t>IPO Matrix / Meth</t>
+          <t>IPO Matrix</t>
         </is>
       </c>
       <c r="G99" s="16" t="inlineStr">
@@ -5912,19 +5919,19 @@
       </c>
       <c r="I99" s="16" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J99" s="17" t="inlineStr">
         <is>
-          <t>test_dataset_stratification.py</t>
+          <t>test_annotation_bounds.py</t>
         </is>
       </c>
     </row>
     <row r="100" ht="22" customHeight="1">
       <c r="A100" s="13" t="inlineStr">
         <is>
-          <t>TASK-AI-DS-02</t>
+          <t>TASK-AI-DS-03</t>
         </is>
       </c>
       <c r="B100" s="13" t="inlineStr">
@@ -5939,17 +5946,17 @@
       </c>
       <c r="D100" s="14" t="inlineStr">
         <is>
-          <t>Whole-Egg YOLO Bounding Box Validator</t>
+          <t>Candling Transillumination Augmentations</t>
         </is>
       </c>
       <c r="E100" s="14" t="inlineStr">
         <is>
-          <t>Verify YOLO darknet format [class_id, x, y, w, h] enclosing whole egg</t>
+          <t>HSV luminance jitter (V +/-20%) and +/-15 deg rotation pipeline</t>
         </is>
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
-          <t>IPO Matrix</t>
+          <t>Chapter 3.2</t>
         </is>
       </c>
       <c r="G100" s="13" t="inlineStr">
@@ -5964,19 +5971,19 @@
       </c>
       <c r="I100" s="13" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P2 - Medium</t>
         </is>
       </c>
       <c r="J100" s="14" t="inlineStr">
         <is>
-          <t>test_annotation_bounds.py</t>
+          <t>test_augmentation_visuals.py</t>
         </is>
       </c>
     </row>
     <row r="101" ht="22" customHeight="1">
       <c r="A101" s="16" t="inlineStr">
         <is>
-          <t>TASK-AI-DS-03</t>
+          <t>TASK-AI-DS-04</t>
         </is>
       </c>
       <c r="B101" s="16" t="inlineStr">
@@ -5991,12 +5998,12 @@
       </c>
       <c r="D101" s="17" t="inlineStr">
         <is>
-          <t>Candling Transillumination Augmentations</t>
+          <t>Dataset Distribution Summary Exporter</t>
         </is>
       </c>
       <c r="E101" s="17" t="inlineStr">
         <is>
-          <t>HSV luminance jitter (V +/-20%) and +/-15 deg rotation pipeline</t>
+          <t>Generate automated Markdown and LaTeX tables of egg counts for manuscript</t>
         </is>
       </c>
       <c r="F101" s="17" t="inlineStr">
@@ -6021,19 +6028,19 @@
       </c>
       <c r="J101" s="17" t="inlineStr">
         <is>
-          <t>test_augmentation_visuals.py</t>
+          <t>export_dataset_table.py</t>
         </is>
       </c>
     </row>
     <row r="102" ht="22" customHeight="1">
       <c r="A102" s="13" t="inlineStr">
         <is>
-          <t>TASK-AI-DS-04</t>
+          <t>TASK-AI-TRN-01</t>
         </is>
       </c>
       <c r="B102" s="13" t="inlineStr">
         <is>
-          <t>Phase 2: Dataset</t>
+          <t>Phase 3: AI Vision</t>
         </is>
       </c>
       <c r="C102" s="14" t="inlineStr">
@@ -6043,17 +6050,17 @@
       </c>
       <c r="D102" s="14" t="inlineStr">
         <is>
-          <t>Dataset Distribution Summary Exporter</t>
+          <t>Ultralytics YOLOv8 Training Script</t>
         </is>
       </c>
       <c r="E102" s="14" t="inlineStr">
         <is>
-          <t>Generate automated Markdown and LaTeX tables of egg counts for manuscript</t>
+          <t>Implement model training pipeline with CIoU + BCE + DFL loss functions</t>
         </is>
       </c>
       <c r="F102" s="14" t="inlineStr">
         <is>
-          <t>Chapter 3.2</t>
+          <t>Methodology 3.3</t>
         </is>
       </c>
       <c r="G102" s="13" t="inlineStr">
@@ -6068,19 +6075,19 @@
       </c>
       <c r="I102" s="13" t="inlineStr">
         <is>
-          <t>P2 - Medium</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J102" s="14" t="inlineStr">
         <is>
-          <t>export_dataset_table.py</t>
+          <t>train_yolov8.py smoke test</t>
         </is>
       </c>
     </row>
     <row r="103" ht="22" customHeight="1">
       <c r="A103" s="16" t="inlineStr">
         <is>
-          <t>TASK-AI-TRN-01</t>
+          <t>TASK-AI-OPT-01</t>
         </is>
       </c>
       <c r="B103" s="16" t="inlineStr">
@@ -6095,17 +6102,17 @@
       </c>
       <c r="D103" s="17" t="inlineStr">
         <is>
-          <t>Ultralytics YOLOv8 Training Script</t>
+          <t>ONNX FP16 Slim Export &amp; Half-Precision Graph</t>
         </is>
       </c>
       <c r="E103" s="17" t="inlineStr">
         <is>
-          <t>Implement model training pipeline with CIoU + BCE + DFL loss functions</t>
+          <t>Convert PyTorch weights to ONNX FP16 slim graph for edge inference</t>
         </is>
       </c>
       <c r="F103" s="17" t="inlineStr">
         <is>
-          <t>Methodology 3.3</t>
+          <t>AGENTS.md Tenet 3</t>
         </is>
       </c>
       <c r="G103" s="16" t="inlineStr">
@@ -6113,26 +6120,26 @@
           <t>Codex</t>
         </is>
       </c>
-      <c r="H103" s="18" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="H103" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I103" s="16" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J103" s="17" t="inlineStr">
         <is>
-          <t>train_yolov8.py smoke test</t>
+          <t>export_onnx.py check</t>
         </is>
       </c>
     </row>
     <row r="104" ht="22" customHeight="1">
       <c r="A104" s="13" t="inlineStr">
         <is>
-          <t>TASK-AI-OPT-01</t>
+          <t>TASK-AI-OPT-02</t>
         </is>
       </c>
       <c r="B104" s="13" t="inlineStr">
@@ -6147,12 +6154,12 @@
       </c>
       <c r="D104" s="14" t="inlineStr">
         <is>
-          <t>ONNX FP16 Slim Export &amp; Half-Precision Graph</t>
+          <t>Production Weights 'edge/models/weights/best.onnx'</t>
         </is>
       </c>
       <c r="E104" s="14" t="inlineStr">
         <is>
-          <t>Convert PyTorch weights to ONNX FP16 slim graph for edge inference</t>
+          <t>Verified production ONNX FP16 weights ready for edge execution</t>
         </is>
       </c>
       <c r="F104" s="14" t="inlineStr">
@@ -6177,14 +6184,14 @@
       </c>
       <c r="J104" s="14" t="inlineStr">
         <is>
-          <t>export_onnx.py check</t>
+          <t>test_inference_engine_and_latency_benchmark</t>
         </is>
       </c>
     </row>
     <row r="105" ht="22" customHeight="1">
       <c r="A105" s="16" t="inlineStr">
         <is>
-          <t>TASK-AI-OPT-02</t>
+          <t>TASK-AI-LAT-01</t>
         </is>
       </c>
       <c r="B105" s="16" t="inlineStr">
@@ -6199,17 +6206,17 @@
       </c>
       <c r="D105" s="17" t="inlineStr">
         <is>
-          <t>Production Weights 'edge/models/weights/best.onnx'</t>
+          <t>Edge Inference Latency Benchmark (&lt;=200ms)</t>
         </is>
       </c>
       <c r="E105" s="17" t="inlineStr">
         <is>
-          <t>Verified production ONNX FP16 weights ready for edge execution</t>
+          <t>Benchmark inference latency ensuring &lt;= 200 ms SLA on edge hardware</t>
         </is>
       </c>
       <c r="F105" s="17" t="inlineStr">
         <is>
-          <t>AGENTS.md Tenet 3</t>
+          <t>Chapter 1 Objectives</t>
         </is>
       </c>
       <c r="G105" s="16" t="inlineStr">
@@ -6236,7 +6243,7 @@
     <row r="106" ht="22" customHeight="1">
       <c r="A106" s="13" t="inlineStr">
         <is>
-          <t>TASK-AI-LAT-01</t>
+          <t>TASK-AI-EVL-01</t>
         </is>
       </c>
       <c r="B106" s="13" t="inlineStr">
@@ -6251,17 +6258,17 @@
       </c>
       <c r="D106" s="14" t="inlineStr">
         <is>
-          <t>Edge Inference Latency Benchmark (&lt;=200ms)</t>
+          <t>Breed Subgroup Metric Evaluator</t>
         </is>
       </c>
       <c r="E106" s="14" t="inlineStr">
         <is>
-          <t>Benchmark inference latency ensuring &lt;= 200 ms SLA on edge hardware</t>
+          <t>Compute Precision, Recall, F1, mAP for IP-Itim, Khaki, and Kayumanggi</t>
         </is>
       </c>
       <c r="F106" s="14" t="inlineStr">
         <is>
-          <t>Chapter 1 Objectives</t>
+          <t>IPO Matrix</t>
         </is>
       </c>
       <c r="G106" s="13" t="inlineStr">
@@ -6269,26 +6276,26 @@
           <t>Codex</t>
         </is>
       </c>
-      <c r="H106" s="15" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="H106" s="18" t="inlineStr">
+        <is>
+          <t>Backlog</t>
         </is>
       </c>
       <c r="I106" s="13" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J106" s="14" t="inlineStr">
         <is>
-          <t>test_inference_engine_and_latency_benchmark</t>
+          <t>test_subgroup_metrics.py</t>
         </is>
       </c>
     </row>
     <row r="107" ht="22" customHeight="1">
       <c r="A107" s="16" t="inlineStr">
         <is>
-          <t>TASK-AI-EVL-01</t>
+          <t>TASK-AI-EVL-02</t>
         </is>
       </c>
       <c r="B107" s="16" t="inlineStr">
@@ -6303,12 +6310,12 @@
       </c>
       <c r="D107" s="17" t="inlineStr">
         <is>
-          <t>Breed Subgroup Metric Evaluator</t>
+          <t>Candling Batch Subgroup Metric Evaluator</t>
         </is>
       </c>
       <c r="E107" s="17" t="inlineStr">
         <is>
-          <t>Compute Precision, Recall, F1, mAP for IP-Itim, Khaki, and Kayumanggi</t>
+          <t>Compute Precision, Recall, F1, mAP across Day 10 batches and genetic groups</t>
         </is>
       </c>
       <c r="F107" s="17" t="inlineStr">
@@ -6340,7 +6347,7 @@
     <row r="108" ht="22" customHeight="1">
       <c r="A108" s="13" t="inlineStr">
         <is>
-          <t>TASK-AI-EVL-02</t>
+          <t>TASK-AI-EVL-03</t>
         </is>
       </c>
       <c r="B108" s="13" t="inlineStr">
@@ -6355,17 +6362,17 @@
       </c>
       <c r="D108" s="14" t="inlineStr">
         <is>
-          <t>Stage Subgroup Metric Evaluator</t>
+          <t>2-Class Confusion Matrix &amp; PR Curve Generator</t>
         </is>
       </c>
       <c r="E108" s="14" t="inlineStr">
         <is>
-          <t>Compute Precision, Recall, F1, mAP across Day 10, Day 18, and Day 25</t>
+          <t>Generate formal 2-class confusion matrix (Fertile, Infertile) for Chapter 4</t>
         </is>
       </c>
       <c r="F108" s="14" t="inlineStr">
         <is>
-          <t>IPO Matrix</t>
+          <t>Chapter 4 Manuscript</t>
         </is>
       </c>
       <c r="G108" s="13" t="inlineStr">
@@ -6380,49 +6387,49 @@
       </c>
       <c r="I108" s="13" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J108" s="14" t="inlineStr">
         <is>
-          <t>test_subgroup_metrics.py</t>
+          <t>generate_confusion_matrix.py</t>
         </is>
       </c>
     </row>
     <row r="109" ht="22" customHeight="1">
       <c r="A109" s="16" t="inlineStr">
         <is>
-          <t>TASK-AI-EVL-03</t>
+          <t>TASK-INT-01</t>
         </is>
       </c>
       <c r="B109" s="16" t="inlineStr">
         <is>
-          <t>Phase 3: AI Vision</t>
+          <t>Phase 5: Integration</t>
         </is>
       </c>
       <c r="C109" s="17" t="inlineStr">
         <is>
-          <t>AI &amp; Data</t>
+          <t>Integration</t>
         </is>
       </c>
       <c r="D109" s="17" t="inlineStr">
         <is>
-          <t>3-Class Confusion Matrix &amp; ROC Generator</t>
+          <t>End-to-End Sorting Pilot Simulation</t>
         </is>
       </c>
       <c r="E109" s="17" t="inlineStr">
         <is>
-          <t>Generate formal confusion matrix and ROC curves for Chapter 4</t>
+          <t>Simulate 50-egg continuous cycle: load -&gt; index -&gt; capture -&gt; predict -&gt; divert -&gt; sync</t>
         </is>
       </c>
       <c r="F109" s="17" t="inlineStr">
         <is>
-          <t>Chapter 4 Manuscript</t>
+          <t>System Flowchart</t>
         </is>
       </c>
       <c r="G109" s="16" t="inlineStr">
         <is>
-          <t>Codex</t>
+          <t>Antigravity / Codex</t>
         </is>
       </c>
       <c r="H109" s="18" t="inlineStr">
@@ -6437,14 +6444,14 @@
       </c>
       <c r="J109" s="17" t="inlineStr">
         <is>
-          <t>generate_confusion_matrix.py</t>
+          <t>test_end_to_end_pilot.py</t>
         </is>
       </c>
     </row>
     <row r="110" ht="22" customHeight="1">
       <c r="A110" s="13" t="inlineStr">
         <is>
-          <t>TASK-INT-01</t>
+          <t>TASK-INT-02</t>
         </is>
       </c>
       <c r="B110" s="13" t="inlineStr">
@@ -6459,17 +6466,17 @@
       </c>
       <c r="D110" s="14" t="inlineStr">
         <is>
-          <t>End-to-End Sorting Pilot Simulation</t>
+          <t>Offline Network Replay Resilience Test</t>
         </is>
       </c>
       <c r="E110" s="14" t="inlineStr">
         <is>
-          <t>Simulate 50-egg continuous cycle: load -&gt; index -&gt; capture -&gt; predict -&gt; divert -&gt; sync</t>
+          <t>Cut network; confirm 100% sorting at edge; reconnect and verify bulk replay</t>
         </is>
       </c>
       <c r="F110" s="14" t="inlineStr">
         <is>
-          <t>System Flowchart</t>
+          <t>AGENTS.md Offline</t>
         </is>
       </c>
       <c r="G110" s="13" t="inlineStr">
@@ -6489,14 +6496,14 @@
       </c>
       <c r="J110" s="14" t="inlineStr">
         <is>
-          <t>test_end_to_end_pilot.py</t>
+          <t>test_offline_network_replay.py</t>
         </is>
       </c>
     </row>
     <row r="111" ht="22" customHeight="1">
       <c r="A111" s="16" t="inlineStr">
         <is>
-          <t>TASK-INT-02</t>
+          <t>TASK-INT-03</t>
         </is>
       </c>
       <c r="B111" s="16" t="inlineStr">
@@ -6511,17 +6518,17 @@
       </c>
       <c r="D111" s="17" t="inlineStr">
         <is>
-          <t>Offline Network Replay Resilience Test</t>
+          <t>Cradle Position Jam Recovery Test</t>
         </is>
       </c>
       <c r="E111" s="17" t="inlineStr">
         <is>
-          <t>Cut network; confirm 100% sorting at edge; reconnect and verify bulk replay</t>
+          <t>Simulate mechanical index slip; verify conveyor pauses and resyncs</t>
         </is>
       </c>
       <c r="F111" s="17" t="inlineStr">
         <is>
-          <t>AGENTS.md Offline</t>
+          <t>System Flowchart Node 16</t>
         </is>
       </c>
       <c r="G111" s="16" t="inlineStr">
@@ -6536,49 +6543,49 @@
       </c>
       <c r="I111" s="16" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J111" s="17" t="inlineStr">
         <is>
-          <t>test_offline_network_replay.py</t>
+          <t>test_cradle_resync_handler.py</t>
         </is>
       </c>
     </row>
     <row r="112" ht="22" customHeight="1">
       <c r="A112" s="13" t="inlineStr">
         <is>
-          <t>TASK-INT-03</t>
+          <t>TASK-EVL-01</t>
         </is>
       </c>
       <c r="B112" s="13" t="inlineStr">
         <is>
-          <t>Phase 5: Integration</t>
+          <t>Phase 6: Evaluation</t>
         </is>
       </c>
       <c r="C112" s="14" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>Evaluation</t>
         </is>
       </c>
       <c r="D112" s="14" t="inlineStr">
         <is>
-          <t>Cradle Position Jam Recovery Test</t>
+          <t>Physical Sorting Accuracy Benchmark</t>
         </is>
       </c>
       <c r="E112" s="14" t="inlineStr">
         <is>
-          <t>Simulate mechanical index slip; verify conveyor pauses and resyncs</t>
+          <t>Run &gt;= 100 physical duck egg trials to measure sorting accuracy rate</t>
         </is>
       </c>
       <c r="F112" s="14" t="inlineStr">
         <is>
-          <t>System Flowchart Node 16</t>
+          <t>Chapter 1 Objectives</t>
         </is>
       </c>
       <c r="G112" s="13" t="inlineStr">
         <is>
-          <t>Antigravity / Codex</t>
+          <t>Antigravity</t>
         </is>
       </c>
       <c r="H112" s="18" t="inlineStr">
@@ -6588,19 +6595,19 @@
       </c>
       <c r="I112" s="13" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J112" s="14" t="inlineStr">
         <is>
-          <t>test_cradle_resync_handler.py</t>
+          <t>Physical trial tally sheet</t>
         </is>
       </c>
     </row>
     <row r="113" ht="22" customHeight="1">
       <c r="A113" s="16" t="inlineStr">
         <is>
-          <t>TASK-EVL-01</t>
+          <t>TASK-EVL-02</t>
         </is>
       </c>
       <c r="B113" s="16" t="inlineStr">
@@ -6615,12 +6622,12 @@
       </c>
       <c r="D113" s="17" t="inlineStr">
         <is>
-          <t>Physical Sorting Accuracy Benchmark</t>
+          <t>System Throughput &amp; Cycle Time Profiling</t>
         </is>
       </c>
       <c r="E113" s="17" t="inlineStr">
         <is>
-          <t>Run &gt;= 100 physical duck egg trials to measure sorting accuracy rate</t>
+          <t>Measure end-to-end cycle time per egg and throughput (eggs/min)</t>
         </is>
       </c>
       <c r="F113" s="17" t="inlineStr">
@@ -6640,44 +6647,44 @@
       </c>
       <c r="I113" s="16" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J113" s="17" t="inlineStr">
         <is>
-          <t>Physical trial tally sheet</t>
+          <t>Kinematics benchmark report</t>
         </is>
       </c>
     </row>
     <row r="114" ht="22" customHeight="1">
       <c r="A114" s="13" t="inlineStr">
         <is>
-          <t>TASK-EVL-02</t>
+          <t>TASK-DEF-01</t>
         </is>
       </c>
       <c r="B114" s="13" t="inlineStr">
         <is>
-          <t>Phase 6: Evaluation</t>
+          <t>Phase 7: Defense</t>
         </is>
       </c>
       <c r="C114" s="14" t="inlineStr">
         <is>
-          <t>Evaluation</t>
+          <t>Defense Prep</t>
         </is>
       </c>
       <c r="D114" s="14" t="inlineStr">
         <is>
-          <t>System Throughput &amp; Cycle Time Profiling</t>
+          <t>Manuscript Chapter 4 (Results &amp; Discussion)</t>
         </is>
       </c>
       <c r="E114" s="14" t="inlineStr">
         <is>
-          <t>Measure end-to-end cycle time per egg and throughput (eggs/min)</t>
+          <t>Draft Chapter 4 using empirical metrics, confusion matrices, latency charts</t>
         </is>
       </c>
       <c r="F114" s="14" t="inlineStr">
         <is>
-          <t>Chapter 1 Objectives</t>
+          <t>Chapter 4</t>
         </is>
       </c>
       <c r="G114" s="13" t="inlineStr">
@@ -6692,19 +6699,19 @@
       </c>
       <c r="I114" s="13" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J114" s="14" t="inlineStr">
         <is>
-          <t>Kinematics benchmark report</t>
+          <t>Manuscript peer review</t>
         </is>
       </c>
     </row>
     <row r="115" ht="22" customHeight="1">
       <c r="A115" s="16" t="inlineStr">
         <is>
-          <t>TASK-DEF-01</t>
+          <t>TASK-DEF-02</t>
         </is>
       </c>
       <c r="B115" s="16" t="inlineStr">
@@ -6719,17 +6726,17 @@
       </c>
       <c r="D115" s="17" t="inlineStr">
         <is>
-          <t>Manuscript Chapter 4 (Results &amp; Discussion)</t>
+          <t>Manuscript Chapter 5 (Conclusions &amp; Recommendations)</t>
         </is>
       </c>
       <c r="E115" s="17" t="inlineStr">
         <is>
-          <t>Draft Chapter 4 using empirical metrics, confusion matrices, latency charts</t>
+          <t>Summarize findings, answer research questions 1-4, formulate recommendations</t>
         </is>
       </c>
       <c r="F115" s="17" t="inlineStr">
         <is>
-          <t>Chapter 4</t>
+          <t>Chapter 5</t>
         </is>
       </c>
       <c r="G115" s="16" t="inlineStr">
@@ -6749,14 +6756,14 @@
       </c>
       <c r="J115" s="17" t="inlineStr">
         <is>
-          <t>Manuscript peer review</t>
+          <t>Adviser review</t>
         </is>
       </c>
     </row>
     <row r="116" ht="22" customHeight="1">
       <c r="A116" s="13" t="inlineStr">
         <is>
-          <t>TASK-DEF-02</t>
+          <t>TASK-DEF-03</t>
         </is>
       </c>
       <c r="B116" s="13" t="inlineStr">
@@ -6766,32 +6773,32 @@
       </c>
       <c r="C116" s="14" t="inlineStr">
         <is>
-          <t>Defense Prep</t>
+          <t>Deployment</t>
         </is>
       </c>
       <c r="D116" s="14" t="inlineStr">
         <is>
-          <t>Manuscript Chapter 5 (Conclusions &amp; Recommendations)</t>
+          <t>1-Click Docker Production Verification</t>
         </is>
       </c>
       <c r="E116" s="14" t="inlineStr">
         <is>
-          <t>Summarize findings, answer research questions 1-4, formulate recommendations</t>
+          <t>Verify docker-compose up for PostgreSQL 16, FastAPI backend, React dashboard</t>
         </is>
       </c>
       <c r="F116" s="14" t="inlineStr">
         <is>
-          <t>Chapter 5</t>
+          <t>docker-compose.yml</t>
         </is>
       </c>
       <c r="G116" s="13" t="inlineStr">
         <is>
-          <t>Antigravity</t>
-        </is>
-      </c>
-      <c r="H116" s="18" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+          <t>Antigravity / Codex</t>
+        </is>
+      </c>
+      <c r="H116" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I116" s="13" t="inlineStr">
@@ -6800,58 +6807,6 @@
         </is>
       </c>
       <c r="J116" s="14" t="inlineStr">
-        <is>
-          <t>Adviser review</t>
-        </is>
-      </c>
-    </row>
-    <row r="117" ht="22" customHeight="1">
-      <c r="A117" s="16" t="inlineStr">
-        <is>
-          <t>TASK-DEF-03</t>
-        </is>
-      </c>
-      <c r="B117" s="16" t="inlineStr">
-        <is>
-          <t>Phase 7: Defense</t>
-        </is>
-      </c>
-      <c r="C117" s="17" t="inlineStr">
-        <is>
-          <t>Deployment</t>
-        </is>
-      </c>
-      <c r="D117" s="17" t="inlineStr">
-        <is>
-          <t>1-Click Docker Production Verification</t>
-        </is>
-      </c>
-      <c r="E117" s="17" t="inlineStr">
-        <is>
-          <t>Verify docker-compose up for PostgreSQL 16, FastAPI backend, React dashboard</t>
-        </is>
-      </c>
-      <c r="F117" s="17" t="inlineStr">
-        <is>
-          <t>docker-compose.yml</t>
-        </is>
-      </c>
-      <c r="G117" s="16" t="inlineStr">
-        <is>
-          <t>Antigravity / Codex</t>
-        </is>
-      </c>
-      <c r="H117" s="15" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="I117" s="16" t="inlineStr">
-        <is>
-          <t>P0 - Critical</t>
-        </is>
-      </c>
-      <c r="J117" s="17" t="inlineStr">
         <is>
           <t>docker-compose config test</t>
         </is>

</xml_diff>

<commit_message>
refactor(backend): enforce Day 10 binary candling contract
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -593,7 +593,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
@@ -634,8 +633,6 @@
         <v/>
       </c>
     </row>
-    <row r="6"/>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
@@ -807,8 +804,6 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -840,7 +835,7 @@
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>4. Strict Architectural Tenets: Zero Firebase (100% FastAPI+PostgreSQL), offline SQLite WAL at edge, strict 2 biological classes (Fertile, Infertile), Day 10 candling, FU branding (#800000).</t>
+          <t>4. Strict Architectural Tenets: Zero Firebase (100% FastAPI+PostgreSQL), offline SQLite WAL at edge, 3 biological classes, FU branding (#800000).</t>
         </is>
       </c>
     </row>
@@ -867,7 +862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J116"/>
+  <dimension ref="A3:J117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -882,8 +877,6 @@
     <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
@@ -1095,32 +1088,32 @@
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-AUTH-01</t>
+          <t>TASK-NEW-SCOPE-01</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Phase 4C: Backend</t>
+          <t>Phase 4: Development</t>
         </is>
       </c>
       <c r="C7" s="17" t="inlineStr">
         <is>
-          <t>Backend API</t>
+          <t>Cross-System</t>
         </is>
       </c>
       <c r="D7" s="17" t="inlineStr">
         <is>
-          <t>POST /api/v1/auth/login</t>
+          <t>Day 10 Binary Domain Refactor</t>
         </is>
       </c>
       <c r="E7" s="17" t="inlineStr">
         <is>
-          <t>JWT authentication endpoint with bcrypt password verification and role extraction</t>
+          <t>Standardize backend, edge, dashboard, firmware, tests, and docs on Day 10 with FERTILE/INFERTILE outcomes</t>
         </is>
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t>Use Case: Worker</t>
+          <t>System-wide contract</t>
         </is>
       </c>
       <c r="G7" s="16" t="inlineStr">
@@ -1140,14 +1133,14 @@
       </c>
       <c r="J7" s="17" t="inlineStr">
         <is>
-          <t>test_login_and_me</t>
+          <t>pytest + npm.cmd run build</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-AUTH-02</t>
+          <t>TASK-BE-AUTH-01</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
@@ -1162,12 +1155,12 @@
       </c>
       <c r="D8" s="14" t="inlineStr">
         <is>
-          <t>GET /api/v1/auth/me</t>
+          <t>POST /api/v1/auth/login</t>
         </is>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>Retrieve current authenticated user profile, permissions, and active status</t>
+          <t>JWT authentication endpoint with bcrypt password verification and role extraction</t>
         </is>
       </c>
       <c r="F8" s="14" t="inlineStr">
@@ -1199,7 +1192,7 @@
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-AUTH-03</t>
+          <t>TASK-BE-AUTH-02</t>
         </is>
       </c>
       <c r="B9" s="16" t="inlineStr">
@@ -1214,17 +1207,17 @@
       </c>
       <c r="D9" s="17" t="inlineStr">
         <is>
-          <t>POST /api/v1/auth/register</t>
+          <t>GET /api/v1/auth/me</t>
         </is>
       </c>
       <c r="E9" s="17" t="inlineStr">
         <is>
-          <t>Account registration endpoint with default Candling Worker role</t>
+          <t>Retrieve current authenticated user profile, permissions, and active status</t>
         </is>
       </c>
       <c r="F9" s="17" t="inlineStr">
         <is>
-          <t>Use Case: Admin</t>
+          <t>Use Case: Worker</t>
         </is>
       </c>
       <c r="G9" s="16" t="inlineStr">
@@ -1239,19 +1232,19 @@
       </c>
       <c r="I9" s="16" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J9" s="17" t="inlineStr">
         <is>
-          <t>test_rbac_and_admin_security_protections</t>
+          <t>test_login_and_me</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-USR-01</t>
+          <t>TASK-BE-AUTH-03</t>
         </is>
       </c>
       <c r="B10" s="13" t="inlineStr">
@@ -1266,12 +1259,12 @@
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>GET /api/v1/users</t>
+          <t>POST /api/v1/auth/register</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>List all system users with role filters (Worker, Supervisor, Admin)</t>
+          <t>Account registration endpoint with default Candling Worker role</t>
         </is>
       </c>
       <c r="F10" s="14" t="inlineStr">
@@ -1303,7 +1296,7 @@
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-USR-02</t>
+          <t>TASK-BE-USR-01</t>
         </is>
       </c>
       <c r="B11" s="16" t="inlineStr">
@@ -1318,12 +1311,12 @@
       </c>
       <c r="D11" s="17" t="inlineStr">
         <is>
-          <t>POST /api/v1/users</t>
+          <t>GET /api/v1/users</t>
         </is>
       </c>
       <c r="E11" s="17" t="inlineStr">
         <is>
-          <t>Admin user creation endpoint with RBAC role assignment</t>
+          <t>List all system users with role filters (Worker, Supervisor, Admin)</t>
         </is>
       </c>
       <c r="F11" s="17" t="inlineStr">
@@ -1355,7 +1348,7 @@
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-USR-03</t>
+          <t>TASK-BE-USR-02</t>
         </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
@@ -1370,12 +1363,12 @@
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>PATCH /api/v1/users/{id}/status</t>
+          <t>POST /api/v1/users</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>Toggle user active/deactivated state to revoke credentials</t>
+          <t>Admin user creation endpoint with RBAC role assignment</t>
         </is>
       </c>
       <c r="F12" s="14" t="inlineStr">
@@ -1407,7 +1400,7 @@
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-USR-04</t>
+          <t>TASK-BE-USR-03</t>
         </is>
       </c>
       <c r="B13" s="16" t="inlineStr">
@@ -1422,17 +1415,17 @@
       </c>
       <c r="D13" s="17" t="inlineStr">
         <is>
-          <t>PATCH /api/v1/users/me/profile</t>
+          <t>PATCH /api/v1/users/{id}/status</t>
         </is>
       </c>
       <c r="E13" s="17" t="inlineStr">
         <is>
-          <t>Allow authenticated user to update their display name and email</t>
+          <t>Toggle user active/deactivated state to revoke credentials</t>
         </is>
       </c>
       <c r="F13" s="17" t="inlineStr">
         <is>
-          <t>Use Case: Worker</t>
+          <t>Use Case: Admin</t>
         </is>
       </c>
       <c r="G13" s="16" t="inlineStr">
@@ -1447,19 +1440,19 @@
       </c>
       <c r="I13" s="16" t="inlineStr">
         <is>
-          <t>P2 - Medium</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J13" s="17" t="inlineStr">
         <is>
-          <t>test_user_profile_and_password_change_flow</t>
+          <t>test_rbac_and_admin_security_protections</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-USR-05</t>
+          <t>TASK-BE-USR-04</t>
         </is>
       </c>
       <c r="B14" s="13" t="inlineStr">
@@ -1474,12 +1467,12 @@
       </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
-          <t>PATCH /api/v1/users/me/password</t>
+          <t>PATCH /api/v1/users/me/profile</t>
         </is>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>Secure password change with old password verification</t>
+          <t>Allow authenticated user to update their display name and email</t>
         </is>
       </c>
       <c r="F14" s="14" t="inlineStr">
@@ -1499,7 +1492,7 @@
       </c>
       <c r="I14" s="13" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P2 - Medium</t>
         </is>
       </c>
       <c r="J14" s="14" t="inlineStr">
@@ -1511,7 +1504,7 @@
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-BAT-01</t>
+          <t>TASK-BE-USR-05</t>
         </is>
       </c>
       <c r="B15" s="16" t="inlineStr">
@@ -1526,17 +1519,17 @@
       </c>
       <c r="D15" s="17" t="inlineStr">
         <is>
-          <t>GET /api/v1/batches</t>
+          <t>PATCH /api/v1/users/me/password</t>
         </is>
       </c>
       <c r="E15" s="17" t="inlineStr">
         <is>
-          <t>List incubation batches with status and genetic group filters</t>
+          <t>Secure password change with old password verification</t>
         </is>
       </c>
       <c r="F15" s="17" t="inlineStr">
         <is>
-          <t>Use Case: Supervisor</t>
+          <t>Use Case: Worker</t>
         </is>
       </c>
       <c r="G15" s="16" t="inlineStr">
@@ -1551,19 +1544,19 @@
       </c>
       <c r="I15" s="16" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J15" s="17" t="inlineStr">
         <is>
-          <t>test_list_batches</t>
+          <t>test_user_profile_and_password_change_flow</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-BAT-02</t>
+          <t>TASK-BE-BAT-01</t>
         </is>
       </c>
       <c r="B16" s="13" t="inlineStr">
@@ -1578,12 +1571,12 @@
       </c>
       <c r="D16" s="14" t="inlineStr">
         <is>
-          <t>GET /api/v1/batches/active</t>
+          <t>GET /api/v1/batches</t>
         </is>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>Retrieve currently active incubator batches needing candling inspection</t>
+          <t>List incubation batches with status and genetic group filters</t>
         </is>
       </c>
       <c r="F16" s="14" t="inlineStr">
@@ -1615,7 +1608,7 @@
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-BAT-03</t>
+          <t>TASK-BE-BAT-02</t>
         </is>
       </c>
       <c r="B17" s="16" t="inlineStr">
@@ -1630,12 +1623,12 @@
       </c>
       <c r="D17" s="17" t="inlineStr">
         <is>
-          <t>POST /api/v1/batches</t>
+          <t>GET /api/v1/batches/active</t>
         </is>
       </c>
       <c r="E17" s="17" t="inlineStr">
         <is>
-          <t>Create new incubation batch specifying breed (Itim/Khaki/Kayumanggi) and egg count</t>
+          <t>Retrieve currently active incubator batches needing candling inspection</t>
         </is>
       </c>
       <c r="F17" s="17" t="inlineStr">
@@ -1660,14 +1653,14 @@
       </c>
       <c r="J17" s="17" t="inlineStr">
         <is>
-          <t>test_batch_analytics_and_milestones</t>
+          <t>test_list_batches</t>
         </is>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-BAT-04</t>
+          <t>TASK-BE-BAT-03</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
@@ -1682,12 +1675,12 @@
       </c>
       <c r="D18" s="14" t="inlineStr">
         <is>
-          <t>GET /api/v1/batches/{id}</t>
+          <t>POST /api/v1/batches</t>
         </is>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>Get detailed batch record with tray matrix slots and current milestone</t>
+          <t>Create new incubation batch specifying breed (Itim/Khaki/Kayumanggi) and egg count</t>
         </is>
       </c>
       <c r="F18" s="14" t="inlineStr">
@@ -1719,7 +1712,7 @@
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-BAT-05</t>
+          <t>TASK-BE-BAT-04</t>
         </is>
       </c>
       <c r="B19" s="16" t="inlineStr">
@@ -1734,12 +1727,12 @@
       </c>
       <c r="D19" s="17" t="inlineStr">
         <is>
-          <t>GET /api/v1/batches/{id}/analytics</t>
+          <t>GET /api/v1/batches/{id}</t>
         </is>
       </c>
       <c r="E19" s="17" t="inlineStr">
         <is>
-          <t>Incubation analytics: fertility rate, mortality curve, penoy salvage total</t>
+          <t>Get detailed batch record with tray matrix slots and current milestone</t>
         </is>
       </c>
       <c r="F19" s="17" t="inlineStr">
@@ -1771,7 +1764,7 @@
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-BAT-06</t>
+          <t>TASK-BE-BAT-05</t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
@@ -1786,12 +1779,12 @@
       </c>
       <c r="D20" s="14" t="inlineStr">
         <is>
-          <t>GET /api/v1/batches/{id}/forecast</t>
+          <t>GET /api/v1/batches/{id}/analytics</t>
         </is>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>Hatch yield forecast calculation based on Day 10 fertility viability rate</t>
+          <t>Incubation analytics: fertility rate, mortality curve, penoy salvage total</t>
         </is>
       </c>
       <c r="F20" s="14" t="inlineStr">
@@ -1811,19 +1804,19 @@
       </c>
       <c r="I20" s="13" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>test_hatch_yield_forecast_and_backup_service</t>
+          <t>test_batch_analytics_and_milestones</t>
         </is>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-BAT-07</t>
+          <t>TASK-BE-BAT-06</t>
         </is>
       </c>
       <c r="B21" s="16" t="inlineStr">
@@ -1838,12 +1831,12 @@
       </c>
       <c r="D21" s="17" t="inlineStr">
         <is>
-          <t>PUT /api/v1/batches/{id}</t>
+          <t>GET /api/v1/batches/{id}/forecast</t>
         </is>
       </c>
       <c r="E21" s="17" t="inlineStr">
         <is>
-          <t>Update batch metadata, notes, and incubator chamber ID</t>
+          <t>Hatch yield forecast based on the Day 10 fertility rate</t>
         </is>
       </c>
       <c r="F21" s="17" t="inlineStr">
@@ -1868,14 +1861,14 @@
       </c>
       <c r="J21" s="17" t="inlineStr">
         <is>
-          <t>test_batch_analytics_and_milestones</t>
+          <t>test_hatch_yield_forecast_and_backup_service</t>
         </is>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-BAT-08</t>
+          <t>TASK-BE-BAT-07</t>
         </is>
       </c>
       <c r="B22" s="13" t="inlineStr">
@@ -1890,12 +1883,12 @@
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>POST /api/v1/batches/{id}/advance-stage</t>
+          <t>PUT /api/v1/batches/{id}</t>
         </is>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>Advance batch milestone: SETTING -&gt; DAY_10 -&gt; HATCHED -&gt; COMPLETED</t>
+          <t>Update batch metadata, notes, and incubator chamber ID</t>
         </is>
       </c>
       <c r="F22" s="14" t="inlineStr">
@@ -1915,7 +1908,7 @@
       </c>
       <c r="I22" s="13" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J22" s="14" t="inlineStr">
@@ -1927,7 +1920,7 @@
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-BAT-09</t>
+          <t>TASK-BE-BAT-08</t>
         </is>
       </c>
       <c r="B23" s="16" t="inlineStr">
@@ -1942,12 +1935,12 @@
       </c>
       <c r="D23" s="17" t="inlineStr">
         <is>
-          <t>POST /api/v1/batches/{id}/finalize-hatch</t>
+          <t>POST /api/v1/batches/{id}/advance-stage</t>
         </is>
       </c>
       <c r="E23" s="17" t="inlineStr">
         <is>
-          <t>Close batch lifecycle and record final hatchling count on Day 28</t>
+          <t>Advance lifecycle: Setting -&gt; Day 10 -&gt; Hatched -&gt; Completed</t>
         </is>
       </c>
       <c r="F23" s="17" t="inlineStr">
@@ -1967,7 +1960,7 @@
       </c>
       <c r="I23" s="16" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J23" s="17" t="inlineStr">
@@ -1979,7 +1972,7 @@
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-BAT-10</t>
+          <t>TASK-BE-BAT-09</t>
         </is>
       </c>
       <c r="B24" s="13" t="inlineStr">
@@ -1994,12 +1987,12 @@
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
-          <t>GET /api/v1/batches/{id}/summary</t>
+          <t>POST /api/v1/batches/{id}/finalize-hatch</t>
         </is>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>Comprehensive batch summary DTO for compliance and audit archiving</t>
+          <t>Close batch lifecycle and record final hatchling count on Day 28</t>
         </is>
       </c>
       <c r="F24" s="14" t="inlineStr">
@@ -2031,7 +2024,7 @@
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-BAT-11</t>
+          <t>TASK-BE-BAT-10</t>
         </is>
       </c>
       <c r="B25" s="16" t="inlineStr">
@@ -2046,17 +2039,17 @@
       </c>
       <c r="D25" s="17" t="inlineStr">
         <is>
-          <t>DELETE /api/v1/batches/{id}</t>
+          <t>GET /api/v1/batches/{id}/summary</t>
         </is>
       </c>
       <c r="E25" s="17" t="inlineStr">
         <is>
-          <t>Soft-delete or purge batch (Admin only protection)</t>
+          <t>Comprehensive batch summary DTO for compliance and audit archiving</t>
         </is>
       </c>
       <c r="F25" s="17" t="inlineStr">
         <is>
-          <t>Use Case: Admin</t>
+          <t>Use Case: Supervisor</t>
         </is>
       </c>
       <c r="G25" s="16" t="inlineStr">
@@ -2071,19 +2064,19 @@
       </c>
       <c r="I25" s="16" t="inlineStr">
         <is>
-          <t>P2 - Medium</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>test_rbac_and_admin_security_protections</t>
+          <t>test_batch_analytics_and_milestones</t>
         </is>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-BAT-12</t>
+          <t>TASK-BE-BAT-11</t>
         </is>
       </c>
       <c r="B26" s="13" t="inlineStr">
@@ -2098,17 +2091,17 @@
       </c>
       <c r="D26" s="14" t="inlineStr">
         <is>
-          <t>POST /api/v1/batches/check-milestones</t>
+          <t>DELETE /api/v1/batches/{id}</t>
         </is>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>Automated background cron to flag batches reaching Day 10 candling milestone</t>
+          <t>Soft-delete or purge batch (Admin only protection)</t>
         </is>
       </c>
       <c r="F26" s="14" t="inlineStr">
         <is>
-          <t>System Flowchart</t>
+          <t>Use Case: Admin</t>
         </is>
       </c>
       <c r="G26" s="13" t="inlineStr">
@@ -2123,19 +2116,19 @@
       </c>
       <c r="I26" s="13" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P2 - Medium</t>
         </is>
       </c>
       <c r="J26" s="14" t="inlineStr">
         <is>
-          <t>test_batch_analytics_and_milestones</t>
+          <t>test_rbac_and_admin_security_protections</t>
         </is>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-SES-01</t>
+          <t>TASK-BE-BAT-12</t>
         </is>
       </c>
       <c r="B27" s="16" t="inlineStr">
@@ -2150,17 +2143,17 @@
       </c>
       <c r="D27" s="17" t="inlineStr">
         <is>
-          <t>GET /api/v1/sessions</t>
+          <t>POST /api/v1/batches/check-milestones</t>
         </is>
       </c>
       <c r="E27" s="17" t="inlineStr">
         <is>
-          <t>List all active and completed edge candling sorting sessions</t>
+          <t>Automated background cron to flag batches reaching Day 10, 18, 25</t>
         </is>
       </c>
       <c r="F27" s="17" t="inlineStr">
         <is>
-          <t>Use Case: Worker</t>
+          <t>System Flowchart</t>
         </is>
       </c>
       <c r="G27" s="16" t="inlineStr">
@@ -2175,19 +2168,19 @@
       </c>
       <c r="I27" s="16" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
-          <t>test_api.py</t>
+          <t>test_batch_analytics_and_milestones</t>
         </is>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-SES-02</t>
+          <t>TASK-BE-SES-01</t>
         </is>
       </c>
       <c r="B28" s="13" t="inlineStr">
@@ -2202,12 +2195,12 @@
       </c>
       <c r="D28" s="14" t="inlineStr">
         <is>
-          <t>POST /api/v1/sessions</t>
+          <t>GET /api/v1/sessions</t>
         </is>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>Start new candling session linked to batch and edge sorter device ID</t>
+          <t>List all active and completed edge candling sorting sessions</t>
         </is>
       </c>
       <c r="F28" s="14" t="inlineStr">
@@ -2239,7 +2232,7 @@
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-SES-03</t>
+          <t>TASK-BE-SES-02</t>
         </is>
       </c>
       <c r="B29" s="16" t="inlineStr">
@@ -2254,12 +2247,12 @@
       </c>
       <c r="D29" s="17" t="inlineStr">
         <is>
-          <t>GET /api/v1/sessions/{id}</t>
+          <t>POST /api/v1/sessions</t>
         </is>
       </c>
       <c r="E29" s="17" t="inlineStr">
         <is>
-          <t>Get session progress: total eggs candled, fertile, infertile counts</t>
+          <t>Start new candling session linked to batch and edge sorter device ID</t>
         </is>
       </c>
       <c r="F29" s="17" t="inlineStr">
@@ -2291,7 +2284,7 @@
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-SES-04</t>
+          <t>TASK-BE-SES-03</t>
         </is>
       </c>
       <c r="B30" s="13" t="inlineStr">
@@ -2306,12 +2299,12 @@
       </c>
       <c r="D30" s="14" t="inlineStr">
         <is>
-          <t>PUT /api/v1/sessions/{id}/end</t>
+          <t>GET /api/v1/sessions/{id}</t>
         </is>
       </c>
       <c r="E30" s="14" t="inlineStr">
         <is>
-          <t>Conclude candling session and trigger batch analytics recalculation</t>
+          <t>Get Day 10 progress: total, fertile, and infertile counts</t>
         </is>
       </c>
       <c r="F30" s="14" t="inlineStr">
@@ -2343,7 +2336,7 @@
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-SCN-01</t>
+          <t>TASK-BE-SES-04</t>
         </is>
       </c>
       <c r="B31" s="16" t="inlineStr">
@@ -2358,17 +2351,17 @@
       </c>
       <c r="D31" s="17" t="inlineStr">
         <is>
-          <t>POST /api/v1/scans/sync</t>
+          <t>PUT /api/v1/sessions/{id}/end</t>
         </is>
       </c>
       <c r="E31" s="17" t="inlineStr">
         <is>
-          <t>Idempotent batch scan sync with ON CONFLICT (scan_id) DO NOTHING</t>
+          <t>Conclude candling session and trigger batch analytics recalculation</t>
         </is>
       </c>
       <c r="F31" s="17" t="inlineStr">
         <is>
-          <t>System Flowchart</t>
+          <t>Use Case: Worker</t>
         </is>
       </c>
       <c r="G31" s="16" t="inlineStr">
@@ -2388,14 +2381,14 @@
       </c>
       <c r="J31" s="17" t="inlineStr">
         <is>
-          <t>test_analytics_overview</t>
+          <t>test_api.py</t>
         </is>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-SCN-02</t>
+          <t>TASK-BE-SCN-01</t>
         </is>
       </c>
       <c r="B32" s="13" t="inlineStr">
@@ -2410,12 +2403,12 @@
       </c>
       <c r="D32" s="14" t="inlineStr">
         <is>
-          <t>POST /api/v1/scans/upload-image</t>
+          <t>POST /api/v1/scans/sync</t>
         </is>
       </c>
       <c r="E32" s="14" t="inlineStr">
         <is>
-          <t>Upload high-res candling frame image associated with scan ID</t>
+          <t>Idempotent batch scan sync with ON CONFLICT (scan_id) DO NOTHING</t>
         </is>
       </c>
       <c r="F32" s="14" t="inlineStr">
@@ -2435,19 +2428,19 @@
       </c>
       <c r="I32" s="13" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J32" s="14" t="inlineStr">
         <is>
-          <t>test_api.py</t>
+          <t>test_analytics_overview</t>
         </is>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-SCN-03</t>
+          <t>TASK-BE-SCN-02</t>
         </is>
       </c>
       <c r="B33" s="16" t="inlineStr">
@@ -2462,17 +2455,17 @@
       </c>
       <c r="D33" s="17" t="inlineStr">
         <is>
-          <t>GET /api/v1/scans</t>
+          <t>POST /api/v1/scans/upload-image</t>
         </is>
       </c>
       <c r="E33" s="17" t="inlineStr">
         <is>
-          <t>Query historical scans with batch_id, stage, class, date filters</t>
+          <t>Upload high-res candling frame image associated with scan ID</t>
         </is>
       </c>
       <c r="F33" s="17" t="inlineStr">
         <is>
-          <t>Use Case: Supervisor</t>
+          <t>System Flowchart</t>
         </is>
       </c>
       <c r="G33" s="16" t="inlineStr">
@@ -2487,7 +2480,7 @@
       </c>
       <c r="I33" s="16" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J33" s="17" t="inlineStr">
@@ -2499,7 +2492,7 @@
     <row r="34" ht="22" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-SCN-04</t>
+          <t>TASK-BE-SCN-03</t>
         </is>
       </c>
       <c r="B34" s="13" t="inlineStr">
@@ -2514,12 +2507,12 @@
       </c>
       <c r="D34" s="14" t="inlineStr">
         <is>
-          <t>GET /api/v1/scans/{id}</t>
+          <t>GET /api/v1/scans</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
         <is>
-          <t>Retrieve single scan record with confidence, bounding box, image URI</t>
+          <t>Query historical scans with batch_id, stage, class, date filters</t>
         </is>
       </c>
       <c r="F34" s="14" t="inlineStr">
@@ -2539,7 +2532,7 @@
       </c>
       <c r="I34" s="13" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J34" s="14" t="inlineStr">
@@ -2551,7 +2544,7 @@
     <row r="35" ht="22" customHeight="1">
       <c r="A35" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-SCN-05</t>
+          <t>TASK-BE-SCN-04</t>
         </is>
       </c>
       <c r="B35" s="16" t="inlineStr">
@@ -2566,17 +2559,17 @@
       </c>
       <c r="D35" s="17" t="inlineStr">
         <is>
-          <t>PATCH /api/v1/scans/{id}/override</t>
+          <t>GET /api/v1/scans/{id}</t>
         </is>
       </c>
       <c r="E35" s="17" t="inlineStr">
         <is>
-          <t>Human-in-the-loop classification override with audit trail logging</t>
+          <t>Retrieve single scan record with confidence, bounding box, image URI</t>
         </is>
       </c>
       <c r="F35" s="17" t="inlineStr">
         <is>
-          <t>System Flowchart Node 10</t>
+          <t>Use Case: Supervisor</t>
         </is>
       </c>
       <c r="G35" s="16" t="inlineStr">
@@ -2591,19 +2584,19 @@
       </c>
       <c r="I35" s="16" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J35" s="17" t="inlineStr">
         <is>
-          <t>test_human_in_the_loop_override_audit_logging</t>
+          <t>test_api.py</t>
         </is>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-ANL-01</t>
+          <t>TASK-BE-SCN-05</t>
         </is>
       </c>
       <c r="B36" s="13" t="inlineStr">
@@ -2618,17 +2611,17 @@
       </c>
       <c r="D36" s="14" t="inlineStr">
         <is>
-          <t>GET /api/v1/analytics/overview</t>
+          <t>PATCH /api/v1/scans/{id}/override</t>
         </is>
       </c>
       <c r="E36" s="14" t="inlineStr">
         <is>
-          <t>Aggregated hatchery statistics (total eggs, fertility rate, cull rate)</t>
+          <t>Human-in-the-loop classification override with audit trail logging</t>
         </is>
       </c>
       <c r="F36" s="14" t="inlineStr">
         <is>
-          <t>Use Case: Supervisor</t>
+          <t>System Flowchart Node 10</t>
         </is>
       </c>
       <c r="G36" s="13" t="inlineStr">
@@ -2648,14 +2641,14 @@
       </c>
       <c r="J36" s="14" t="inlineStr">
         <is>
-          <t>test_analytics_overview</t>
+          <t>test_human_in_the_loop_override_audit_logging</t>
         </is>
       </c>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-ANL-02</t>
+          <t>TASK-BE-ANL-01</t>
         </is>
       </c>
       <c r="B37" s="16" t="inlineStr">
@@ -2670,17 +2663,17 @@
       </c>
       <c r="D37" s="17" t="inlineStr">
         <is>
-          <t>GET /api/v1/analytics/breed-comparison</t>
+          <t>GET /api/v1/analytics/overview</t>
         </is>
       </c>
       <c r="E37" s="17" t="inlineStr">
         <is>
-          <t>Disaggregated analytics comparing IP-Itim vs IP-Khaki vs IP-Kayumanggi</t>
+          <t>Aggregated hatchery statistics (total eggs, fertility rate, cull rate)</t>
         </is>
       </c>
       <c r="F37" s="17" t="inlineStr">
         <is>
-          <t>Methodology 3.1</t>
+          <t>Use Case: Supervisor</t>
         </is>
       </c>
       <c r="G37" s="16" t="inlineStr">
@@ -2695,7 +2688,7 @@
       </c>
       <c r="I37" s="16" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J37" s="17" t="inlineStr">
@@ -2707,7 +2700,7 @@
     <row r="38" ht="22" customHeight="1">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-ANL-03</t>
+          <t>TASK-BE-ANL-02</t>
         </is>
       </c>
       <c r="B38" s="13" t="inlineStr">
@@ -2722,17 +2715,17 @@
       </c>
       <c r="D38" s="14" t="inlineStr">
         <is>
-          <t>GET /api/v1/analytics/mortality-trends</t>
+          <t>GET /api/v1/analytics/breed-comparison</t>
         </is>
       </c>
       <c r="E38" s="14" t="inlineStr">
         <is>
-          <t>Longitudinal fertility and cull tracking across historical batches</t>
+          <t>Disaggregated analytics comparing IP-Itim vs IP-Khaki vs IP-Kayumanggi</t>
         </is>
       </c>
       <c r="F38" s="14" t="inlineStr">
         <is>
-          <t>Use Case: Supervisor</t>
+          <t>Methodology 3.1</t>
         </is>
       </c>
       <c r="G38" s="13" t="inlineStr">
@@ -2752,14 +2745,14 @@
       </c>
       <c r="J38" s="14" t="inlineStr">
         <is>
-          <t>test_mortality_progression</t>
+          <t>test_analytics_overview</t>
         </is>
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-ANL-04</t>
+          <t>TASK-BE-ANL-03</t>
         </is>
       </c>
       <c r="B39" s="16" t="inlineStr">
@@ -2774,17 +2767,17 @@
       </c>
       <c r="D39" s="17" t="inlineStr">
         <is>
-          <t>GET /api/v1/analytics/mortality-progression</t>
+          <t>GET /api/v1/analytics/mortality-trends</t>
         </is>
       </c>
       <c r="E39" s="17" t="inlineStr">
         <is>
-          <t>Loss analysis and commercial Penoy recovery on Day 10</t>
+          <t>Longitudinal mortality tracking across batches and candling stages</t>
         </is>
       </c>
       <c r="F39" s="17" t="inlineStr">
         <is>
-          <t>Methodology 3.1</t>
+          <t>Use Case: Supervisor</t>
         </is>
       </c>
       <c r="G39" s="16" t="inlineStr">
@@ -2811,7 +2804,7 @@
     <row r="40" ht="22" customHeight="1">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-ANL-05</t>
+          <t>TASK-BE-ANL-04</t>
         </is>
       </c>
       <c r="B40" s="13" t="inlineStr">
@@ -2826,17 +2819,17 @@
       </c>
       <c r="D40" s="14" t="inlineStr">
         <is>
-          <t>GET /api/v1/analytics/economic-yield</t>
+          <t>GET /api/v1/analytics/mortality-progression</t>
         </is>
       </c>
       <c r="E40" s="14" t="inlineStr">
         <is>
-          <t>Day 10 Penoy salvage revenue (Count * P14.00) &amp; thermal energy savings</t>
+          <t>Day 10 cull analysis by breed</t>
         </is>
       </c>
       <c r="F40" s="14" t="inlineStr">
         <is>
-          <t>AGENTS.md Tenet 3</t>
+          <t>Methodology 3.1</t>
         </is>
       </c>
       <c r="G40" s="13" t="inlineStr">
@@ -2851,19 +2844,19 @@
       </c>
       <c r="I40" s="13" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J40" s="14" t="inlineStr">
         <is>
-          <t>test_analytics_economic_yield</t>
+          <t>test_mortality_progression</t>
         </is>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
       <c r="A41" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-REP-01</t>
+          <t>TASK-BE-ANL-05</t>
         </is>
       </c>
       <c r="B41" s="16" t="inlineStr">
@@ -2878,17 +2871,17 @@
       </c>
       <c r="D41" s="17" t="inlineStr">
         <is>
-          <t>GET /api/v1/reports/batch/{id}/csv</t>
+          <t>GET /api/v1/analytics/economic-yield</t>
         </is>
       </c>
       <c r="E41" s="17" t="inlineStr">
         <is>
-          <t>Export CSV spreadsheet containing detailed scan log for batch</t>
+          <t>Day 10 Penoy salvage revenue (Count * P14.00) &amp; thermal energy savings</t>
         </is>
       </c>
       <c r="F41" s="17" t="inlineStr">
         <is>
-          <t>Use Case: Supervisor</t>
+          <t>AGENTS.md Tenet 3</t>
         </is>
       </c>
       <c r="G41" s="16" t="inlineStr">
@@ -2903,19 +2896,19 @@
       </c>
       <c r="I41" s="16" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J41" s="17" t="inlineStr">
         <is>
-          <t>test_pdf_and_csv_reports</t>
+          <t>test_analytics_economic_yield</t>
         </is>
       </c>
     </row>
     <row r="42" ht="22" customHeight="1">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-REP-02</t>
+          <t>TASK-BE-REP-01</t>
         </is>
       </c>
       <c r="B42" s="13" t="inlineStr">
@@ -2930,12 +2923,12 @@
       </c>
       <c r="D42" s="14" t="inlineStr">
         <is>
-          <t>GET /api/v1/reports/batch/{id}/pdf</t>
+          <t>GET /api/v1/reports/batch/{id}/csv</t>
         </is>
       </c>
       <c r="E42" s="14" t="inlineStr">
         <is>
-          <t>Generate official Foundation University formatted PDF compliance report</t>
+          <t>Export CSV spreadsheet containing detailed scan log for batch</t>
         </is>
       </c>
       <c r="F42" s="14" t="inlineStr">
@@ -2955,7 +2948,7 @@
       </c>
       <c r="I42" s="13" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J42" s="14" t="inlineStr">
@@ -2967,7 +2960,7 @@
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-DEV-01</t>
+          <t>TASK-BE-REP-02</t>
         </is>
       </c>
       <c r="B43" s="16" t="inlineStr">
@@ -2982,17 +2975,17 @@
       </c>
       <c r="D43" s="17" t="inlineStr">
         <is>
-          <t>GET /api/v1/devices</t>
+          <t>GET /api/v1/reports/batch/{id}/pdf</t>
         </is>
       </c>
       <c r="E43" s="17" t="inlineStr">
         <is>
-          <t>List registered edge sorter hardware rigs with online/offline status</t>
+          <t>Generate official Foundation University formatted PDF compliance report</t>
         </is>
       </c>
       <c r="F43" s="17" t="inlineStr">
         <is>
-          <t>Use Case: Admin</t>
+          <t>Use Case: Supervisor</t>
         </is>
       </c>
       <c r="G43" s="16" t="inlineStr">
@@ -3007,19 +3000,19 @@
       </c>
       <c r="I43" s="16" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J43" s="17" t="inlineStr">
         <is>
-          <t>test_api.py</t>
+          <t>test_pdf_and_csv_reports</t>
         </is>
       </c>
     </row>
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-DEV-02</t>
+          <t>TASK-BE-DEV-01</t>
         </is>
       </c>
       <c r="B44" s="13" t="inlineStr">
@@ -3034,12 +3027,12 @@
       </c>
       <c r="D44" s="14" t="inlineStr">
         <is>
-          <t>POST /api/v1/devices/register</t>
+          <t>GET /api/v1/devices</t>
         </is>
       </c>
       <c r="E44" s="14" t="inlineStr">
         <is>
-          <t>Register new ESP32 / Raspberry Pi edge node with MAC &amp; station ID</t>
+          <t>List registered edge sorter hardware rigs with online/offline status</t>
         </is>
       </c>
       <c r="F44" s="14" t="inlineStr">
@@ -3071,7 +3064,7 @@
     <row r="45" ht="22" customHeight="1">
       <c r="A45" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-DEV-03</t>
+          <t>TASK-BE-DEV-02</t>
         </is>
       </c>
       <c r="B45" s="16" t="inlineStr">
@@ -3086,12 +3079,12 @@
       </c>
       <c r="D45" s="17" t="inlineStr">
         <is>
-          <t>POST /api/v1/devices/{id}/heartbeat</t>
+          <t>POST /api/v1/devices/register</t>
         </is>
       </c>
       <c r="E45" s="17" t="inlineStr">
         <is>
-          <t>Edge node heartbeat ping transmitting status, temperature, and FPS</t>
+          <t>Register new ESP32 / Raspberry Pi edge node with MAC &amp; station ID</t>
         </is>
       </c>
       <c r="F45" s="17" t="inlineStr">
@@ -3123,7 +3116,7 @@
     <row r="46" ht="22" customHeight="1">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-SET-01</t>
+          <t>TASK-BE-DEV-03</t>
         </is>
       </c>
       <c r="B46" s="13" t="inlineStr">
@@ -3138,12 +3131,12 @@
       </c>
       <c r="D46" s="14" t="inlineStr">
         <is>
-          <t>GET /api/v1/settings</t>
+          <t>POST /api/v1/devices/{id}/heartbeat</t>
         </is>
       </c>
       <c r="E46" s="14" t="inlineStr">
         <is>
-          <t>Fetch system settings (penoy price P14, confidence threshold, sync interval)</t>
+          <t>Edge node heartbeat ping transmitting status, temperature, and FPS</t>
         </is>
       </c>
       <c r="F46" s="14" t="inlineStr">
@@ -3168,14 +3161,14 @@
       </c>
       <c r="J46" s="14" t="inlineStr">
         <is>
-          <t>test_settings_endpoint</t>
+          <t>test_api.py</t>
         </is>
       </c>
     </row>
     <row r="47" ht="22" customHeight="1">
       <c r="A47" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-SET-02</t>
+          <t>TASK-BE-SET-01</t>
         </is>
       </c>
       <c r="B47" s="16" t="inlineStr">
@@ -3190,12 +3183,12 @@
       </c>
       <c r="D47" s="17" t="inlineStr">
         <is>
-          <t>PUT /api/v1/settings</t>
+          <t>GET /api/v1/settings</t>
         </is>
       </c>
       <c r="E47" s="17" t="inlineStr">
         <is>
-          <t>Update system settings with admin validation</t>
+          <t>Fetch system settings (penoy price P14, confidence threshold, sync interval)</t>
         </is>
       </c>
       <c r="F47" s="17" t="inlineStr">
@@ -3227,7 +3220,7 @@
     <row r="48" ht="22" customHeight="1">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-SET-03</t>
+          <t>TASK-BE-SET-02</t>
         </is>
       </c>
       <c r="B48" s="13" t="inlineStr">
@@ -3242,17 +3235,17 @@
       </c>
       <c r="D48" s="14" t="inlineStr">
         <is>
-          <t>POST /api/v1/settings/backups/create</t>
+          <t>PUT /api/v1/settings</t>
         </is>
       </c>
       <c r="E48" s="14" t="inlineStr">
         <is>
-          <t>Trigger compressed JSON.GZ snapshot of PostgreSQL database</t>
+          <t>Update system settings with admin validation</t>
         </is>
       </c>
       <c r="F48" s="14" t="inlineStr">
         <is>
-          <t>AGENTS.md Tenet 1</t>
+          <t>Use Case: Admin</t>
         </is>
       </c>
       <c r="G48" s="13" t="inlineStr">
@@ -3272,14 +3265,14 @@
       </c>
       <c r="J48" s="14" t="inlineStr">
         <is>
-          <t>test_hatch_yield_forecast_and_backup_service</t>
+          <t>test_settings_endpoint</t>
         </is>
       </c>
     </row>
     <row r="49" ht="22" customHeight="1">
       <c r="A49" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-SET-04</t>
+          <t>TASK-BE-SET-03</t>
         </is>
       </c>
       <c r="B49" s="16" t="inlineStr">
@@ -3294,17 +3287,17 @@
       </c>
       <c r="D49" s="17" t="inlineStr">
         <is>
-          <t>GET /api/v1/settings/backups</t>
+          <t>POST /api/v1/settings/backups/create</t>
         </is>
       </c>
       <c r="E49" s="17" t="inlineStr">
         <is>
-          <t>List available database backup archive files</t>
+          <t>Trigger compressed JSON.GZ snapshot of PostgreSQL database</t>
         </is>
       </c>
       <c r="F49" s="17" t="inlineStr">
         <is>
-          <t>Use Case: Admin</t>
+          <t>AGENTS.md Tenet 1</t>
         </is>
       </c>
       <c r="G49" s="16" t="inlineStr">
@@ -3319,7 +3312,7 @@
       </c>
       <c r="I49" s="16" t="inlineStr">
         <is>
-          <t>P2 - Medium</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J49" s="17" t="inlineStr">
@@ -3331,7 +3324,7 @@
     <row r="50" ht="22" customHeight="1">
       <c r="A50" s="13" t="inlineStr">
         <is>
-          <t>TASK-BE-SET-05</t>
+          <t>TASK-BE-SET-04</t>
         </is>
       </c>
       <c r="B50" s="13" t="inlineStr">
@@ -3346,12 +3339,12 @@
       </c>
       <c r="D50" s="14" t="inlineStr">
         <is>
-          <t>GET /api/v1/settings/backups/{file}/download</t>
+          <t>GET /api/v1/settings/backups</t>
         </is>
       </c>
       <c r="E50" s="14" t="inlineStr">
         <is>
-          <t>Secure endpoint to download encrypted database backup</t>
+          <t>List available database backup archive files</t>
         </is>
       </c>
       <c r="F50" s="14" t="inlineStr">
@@ -3383,7 +3376,7 @@
     <row r="51" ht="22" customHeight="1">
       <c r="A51" s="16" t="inlineStr">
         <is>
-          <t>TASK-BE-AUD-01</t>
+          <t>TASK-BE-SET-05</t>
         </is>
       </c>
       <c r="B51" s="16" t="inlineStr">
@@ -3398,12 +3391,12 @@
       </c>
       <c r="D51" s="17" t="inlineStr">
         <is>
-          <t>GET /api/v1/audit_logs</t>
+          <t>GET /api/v1/settings/backups/{file}/download</t>
         </is>
       </c>
       <c r="E51" s="17" t="inlineStr">
         <is>
-          <t>Query immutable system audit trail with user and timestamp filters</t>
+          <t>Secure endpoint to download encrypted database backup</t>
         </is>
       </c>
       <c r="F51" s="17" t="inlineStr">
@@ -3423,44 +3416,44 @@
       </c>
       <c r="I51" s="16" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P2 - Medium</t>
         </is>
       </c>
       <c r="J51" s="17" t="inlineStr">
         <is>
-          <t>test_human_in_the_loop_override_audit_logging</t>
+          <t>test_hatch_yield_forecast_and_backup_service</t>
         </is>
       </c>
     </row>
     <row r="52" ht="22" customHeight="1">
       <c r="A52" s="13" t="inlineStr">
         <is>
-          <t>TASK-EDGE-CAM-01</t>
+          <t>TASK-BE-AUD-01</t>
         </is>
       </c>
       <c r="B52" s="13" t="inlineStr">
         <is>
-          <t>Phase 4B: Edge App</t>
+          <t>Phase 4C: Backend</t>
         </is>
       </c>
       <c r="C52" s="14" t="inlineStr">
         <is>
-          <t>Edge CV</t>
+          <t>Backend API</t>
         </is>
       </c>
       <c r="D52" s="14" t="inlineStr">
         <is>
-          <t>Multi-Threaded Circular Frame Grabber</t>
+          <t>GET /api/v1/audit_logs</t>
         </is>
       </c>
       <c r="E52" s="14" t="inlineStr">
         <is>
-          <t>Thread 1: OpenCV DirectShow/V4L2 continuous circular buffer drain</t>
+          <t>Query immutable system audit trail with user and timestamp filters</t>
         </is>
       </c>
       <c r="F52" s="14" t="inlineStr">
         <is>
-          <t>AGENTS.md Edge</t>
+          <t>Use Case: Admin</t>
         </is>
       </c>
       <c r="G52" s="13" t="inlineStr">
@@ -3480,14 +3473,14 @@
       </c>
       <c r="J52" s="14" t="inlineStr">
         <is>
-          <t>test_camera_mock_generation_and_lifecycle</t>
+          <t>test_human_in_the_loop_override_audit_logging</t>
         </is>
       </c>
     </row>
     <row r="53" ht="22" customHeight="1">
       <c r="A53" s="16" t="inlineStr">
         <is>
-          <t>TASK-EDGE-CAM-02</t>
+          <t>TASK-EDGE-CAM-01</t>
         </is>
       </c>
       <c r="B53" s="16" t="inlineStr">
@@ -3502,12 +3495,12 @@
       </c>
       <c r="D53" s="17" t="inlineStr">
         <is>
-          <t>Camera Disconnect Recovery &amp; Mock Mode</t>
+          <t>Multi-Threaded Circular Frame Grabber</t>
         </is>
       </c>
       <c r="E53" s="17" t="inlineStr">
         <is>
-          <t>Auto-reconnect USB camera and generate mock frames for offline dev</t>
+          <t>Thread 1: OpenCV DirectShow/V4L2 continuous circular buffer drain</t>
         </is>
       </c>
       <c r="F53" s="17" t="inlineStr">
@@ -3527,7 +3520,7 @@
       </c>
       <c r="I53" s="16" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J53" s="17" t="inlineStr">
@@ -3539,7 +3532,7 @@
     <row r="54" ht="22" customHeight="1">
       <c r="A54" s="13" t="inlineStr">
         <is>
-          <t>TASK-EDGE-AI-01</t>
+          <t>TASK-EDGE-CAM-02</t>
         </is>
       </c>
       <c r="B54" s="13" t="inlineStr">
@@ -3554,17 +3547,17 @@
       </c>
       <c r="D54" s="14" t="inlineStr">
         <is>
-          <t>ONNX Runtime FP16 Inference Engine</t>
+          <t>Camera Disconnect Recovery &amp; Mock Mode</t>
         </is>
       </c>
       <c r="E54" s="14" t="inlineStr">
         <is>
-          <t>Thread 2: ONNX Runtime execution provider running quantized YOLOv8</t>
+          <t>Auto-reconnect USB camera and generate mock frames for offline dev</t>
         </is>
       </c>
       <c r="F54" s="14" t="inlineStr">
         <is>
-          <t>System Flowchart Node 8</t>
+          <t>AGENTS.md Edge</t>
         </is>
       </c>
       <c r="G54" s="13" t="inlineStr">
@@ -3579,19 +3572,19 @@
       </c>
       <c r="I54" s="13" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J54" s="14" t="inlineStr">
         <is>
-          <t>test_inference_engine_and_latency_benchmark</t>
+          <t>test_camera_mock_generation_and_lifecycle</t>
         </is>
       </c>
     </row>
     <row r="55" ht="22" customHeight="1">
       <c r="A55" s="16" t="inlineStr">
         <is>
-          <t>TASK-EDGE-AI-02</t>
+          <t>TASK-EDGE-AI-01</t>
         </is>
       </c>
       <c r="B55" s="16" t="inlineStr">
@@ -3606,17 +3599,17 @@
       </c>
       <c r="D55" s="17" t="inlineStr">
         <is>
-          <t>Geometric Aspect-Ratio &amp; Centering Gate</t>
+          <t>ONNX Runtime FP16 Inference Engine</t>
         </is>
       </c>
       <c r="E55" s="17" t="inlineStr">
         <is>
-          <t>Enforce 0.65 &lt;= Aspect Ratio &lt;= 1.45 to prevent classifying non-egg objects</t>
+          <t>Thread 2: ONNX Runtime execution provider running quantized YOLOv8</t>
         </is>
       </c>
       <c r="F55" s="17" t="inlineStr">
         <is>
-          <t>AGENTS.md Edge</t>
+          <t>System Flowchart Node 8</t>
         </is>
       </c>
       <c r="G55" s="16" t="inlineStr">
@@ -3631,19 +3624,19 @@
       </c>
       <c r="I55" s="16" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J55" s="17" t="inlineStr">
         <is>
-          <t>test_candling_heuristics_and_vascularization</t>
+          <t>test_inference_engine_and_latency_benchmark</t>
         </is>
       </c>
     </row>
     <row r="56" ht="22" customHeight="1">
       <c r="A56" s="13" t="inlineStr">
         <is>
-          <t>TASK-EDGE-AI-03</t>
+          <t>TASK-EDGE-AI-02</t>
         </is>
       </c>
       <c r="B56" s="13" t="inlineStr">
@@ -3658,12 +3651,12 @@
       </c>
       <c r="D56" s="14" t="inlineStr">
         <is>
-          <t>Model Cache Warmup Routine</t>
+          <t>Geometric Aspect-Ratio &amp; Centering Gate</t>
         </is>
       </c>
       <c r="E56" s="14" t="inlineStr">
         <is>
-          <t>Execute 3 dummy passes on startup to eliminate first-frame latency spikes</t>
+          <t>Enforce 0.65 &lt;= Aspect Ratio &lt;= 1.45 to prevent classifying non-egg objects</t>
         </is>
       </c>
       <c r="F56" s="14" t="inlineStr">
@@ -3688,14 +3681,14 @@
       </c>
       <c r="J56" s="14" t="inlineStr">
         <is>
-          <t>test_inference_engine_and_latency_benchmark</t>
+          <t>test_candling_heuristics_and_vascularization</t>
         </is>
       </c>
     </row>
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="16" t="inlineStr">
         <is>
-          <t>TASK-EDGE-HEU-01</t>
+          <t>TASK-EDGE-AI-03</t>
         </is>
       </c>
       <c r="B57" s="16" t="inlineStr">
@@ -3710,17 +3703,17 @@
       </c>
       <c r="D57" s="17" t="inlineStr">
         <is>
-          <t>HSV Candling Luminance Analyzer</t>
+          <t>Model Cache Warmup Routine</t>
         </is>
       </c>
       <c r="E57" s="17" t="inlineStr">
         <is>
-          <t>Analyze internal light transmission across yolk/albumin regions</t>
+          <t>Execute 3 dummy passes on startup to eliminate first-frame latency spikes</t>
         </is>
       </c>
       <c r="F57" s="17" t="inlineStr">
         <is>
-          <t>System Flowchart Node 7</t>
+          <t>AGENTS.md Edge</t>
         </is>
       </c>
       <c r="G57" s="16" t="inlineStr">
@@ -3740,14 +3733,14 @@
       </c>
       <c r="J57" s="17" t="inlineStr">
         <is>
-          <t>test_candling_heuristics_and_vascularization</t>
+          <t>test_inference_engine_and_latency_benchmark</t>
         </is>
       </c>
     </row>
     <row r="58" ht="22" customHeight="1">
       <c r="A58" s="13" t="inlineStr">
         <is>
-          <t>TASK-EDGE-HEU-02</t>
+          <t>TASK-EDGE-HEU-01</t>
         </is>
       </c>
       <c r="B58" s="13" t="inlineStr">
@@ -3762,17 +3755,17 @@
       </c>
       <c r="D58" s="14" t="inlineStr">
         <is>
-          <t>Vascular Vein &amp; Blood Ring Heuristics</t>
+          <t>HSV Candling Luminance Analyzer</t>
         </is>
       </c>
       <c r="E58" s="14" t="inlineStr">
         <is>
-          <t>Auxiliary edge detector verifying spider blood veins vs necrotic ring</t>
+          <t>Analyze internal light transmission across yolk/albumin regions</t>
         </is>
       </c>
       <c r="F58" s="14" t="inlineStr">
         <is>
-          <t>System Flowchart Node 8</t>
+          <t>System Flowchart Node 7</t>
         </is>
       </c>
       <c r="G58" s="13" t="inlineStr">
@@ -3799,7 +3792,7 @@
     <row r="59" ht="22" customHeight="1">
       <c r="A59" s="16" t="inlineStr">
         <is>
-          <t>TASK-EDGE-DB-01</t>
+          <t>TASK-EDGE-HEU-02</t>
         </is>
       </c>
       <c r="B59" s="16" t="inlineStr">
@@ -3814,17 +3807,17 @@
       </c>
       <c r="D59" s="17" t="inlineStr">
         <is>
-          <t>Local SQLite WAL Mode Store</t>
+          <t>Vascular Vein &amp; Blood Ring Heuristics</t>
         </is>
       </c>
       <c r="E59" s="17" t="inlineStr">
         <is>
-          <t>Thread 4: Local scan persistence with PRAGMA journal_mode = WAL;</t>
+          <t>Auxiliary edge detector verifying spider blood veins vs necrotic ring</t>
         </is>
       </c>
       <c r="F59" s="17" t="inlineStr">
         <is>
-          <t>AGENTS.md Edge</t>
+          <t>System Flowchart Node 8</t>
         </is>
       </c>
       <c r="G59" s="16" t="inlineStr">
@@ -3839,19 +3832,19 @@
       </c>
       <c r="I59" s="16" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J59" s="17" t="inlineStr">
         <is>
-          <t>test_local_sqlite_wal_and_queue_diagnostics</t>
+          <t>test_candling_heuristics_and_vascularization</t>
         </is>
       </c>
     </row>
     <row r="60" ht="22" customHeight="1">
       <c r="A60" s="13" t="inlineStr">
         <is>
-          <t>TASK-EDGE-DB-02</t>
+          <t>TASK-EDGE-DB-01</t>
         </is>
       </c>
       <c r="B60" s="13" t="inlineStr">
@@ -3866,12 +3859,12 @@
       </c>
       <c r="D60" s="14" t="inlineStr">
         <is>
-          <t>Unsynced Scan FIFO Queue Manager</t>
+          <t>Local SQLite WAL Mode Store</t>
         </is>
       </c>
       <c r="E60" s="14" t="inlineStr">
         <is>
-          <t>Track unsynced scans and handle exponential backoff retry</t>
+          <t>Thread 4: Local scan persistence with PRAGMA journal_mode = WAL;</t>
         </is>
       </c>
       <c r="F60" s="14" t="inlineStr">
@@ -3903,7 +3896,7 @@
     <row r="61" ht="22" customHeight="1">
       <c r="A61" s="16" t="inlineStr">
         <is>
-          <t>TASK-EDGE-SYN-01</t>
+          <t>TASK-EDGE-DB-02</t>
         </is>
       </c>
       <c r="B61" s="16" t="inlineStr">
@@ -3918,17 +3911,17 @@
       </c>
       <c r="D61" s="17" t="inlineStr">
         <is>
-          <t>Background REST HTTP Sync Worker</t>
+          <t>Unsynced Scan FIFO Queue Manager</t>
         </is>
       </c>
       <c r="E61" s="17" t="inlineStr">
         <is>
-          <t>Non-blocking background HTTP client transmitting batches of 50 scans</t>
+          <t>Track unsynced scans and handle exponential backoff retry</t>
         </is>
       </c>
       <c r="F61" s="17" t="inlineStr">
         <is>
-          <t>System Flowchart Node 13</t>
+          <t>AGENTS.md Edge</t>
         </is>
       </c>
       <c r="G61" s="16" t="inlineStr">
@@ -3948,14 +3941,14 @@
       </c>
       <c r="J61" s="17" t="inlineStr">
         <is>
-          <t>test_sync_worker_diagnostics</t>
+          <t>test_local_sqlite_wal_and_queue_diagnostics</t>
         </is>
       </c>
     </row>
     <row r="62" ht="22" customHeight="1">
       <c r="A62" s="13" t="inlineStr">
         <is>
-          <t>TASK-EDGE-SYN-02</t>
+          <t>TASK-EDGE-SYN-01</t>
         </is>
       </c>
       <c r="B62" s="13" t="inlineStr">
@@ -3970,17 +3963,17 @@
       </c>
       <c r="D62" s="14" t="inlineStr">
         <is>
-          <t>Local CSV Session Exporter</t>
+          <t>Background REST HTTP Sync Worker</t>
         </is>
       </c>
       <c r="E62" s="14" t="inlineStr">
         <is>
-          <t>Emergency offline CSV exporter saving session records to local USB drive</t>
+          <t>Non-blocking background HTTP client transmitting batches of 50 scans</t>
         </is>
       </c>
       <c r="F62" s="14" t="inlineStr">
         <is>
-          <t>AGENTS.md Offline</t>
+          <t>System Flowchart Node 13</t>
         </is>
       </c>
       <c r="G62" s="13" t="inlineStr">
@@ -3995,19 +3988,19 @@
       </c>
       <c r="I62" s="13" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J62" s="14" t="inlineStr">
         <is>
-          <t>test_csv_session_export</t>
+          <t>test_sync_worker_diagnostics</t>
         </is>
       </c>
     </row>
     <row r="63" ht="22" customHeight="1">
       <c r="A63" s="16" t="inlineStr">
         <is>
-          <t>TASK-EDGE-SER-01</t>
+          <t>TASK-EDGE-SYN-02</t>
         </is>
       </c>
       <c r="B63" s="16" t="inlineStr">
@@ -4022,17 +4015,17 @@
       </c>
       <c r="D63" s="17" t="inlineStr">
         <is>
-          <t>PySerial ESP32 UART Driver</t>
+          <t>Local CSV Session Exporter</t>
         </is>
       </c>
       <c r="E63" s="17" t="inlineStr">
         <is>
-          <t>Thread 3: Non-blocking serial worker communicating at 115200 baud</t>
+          <t>Emergency offline CSV exporter saving session records to local USB drive</t>
         </is>
       </c>
       <c r="F63" s="17" t="inlineStr">
         <is>
-          <t>System Flowchart Node 17</t>
+          <t>AGENTS.md Offline</t>
         </is>
       </c>
       <c r="G63" s="16" t="inlineStr">
@@ -4047,19 +4040,19 @@
       </c>
       <c r="I63" s="16" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J63" s="17" t="inlineStr">
         <is>
-          <t>test_esp32_serial_mock_and_motor_commands</t>
+          <t>test_csv_session_export</t>
         </is>
       </c>
     </row>
     <row r="64" ht="22" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
         <is>
-          <t>TASK-EDGE-SER-02</t>
+          <t>TASK-EDGE-SER-01</t>
         </is>
       </c>
       <c r="B64" s="13" t="inlineStr">
@@ -4074,17 +4067,17 @@
       </c>
       <c r="D64" s="14" t="inlineStr">
         <is>
-          <t>Serial Mock Driver for Hardware-Free Dev</t>
+          <t>PySerial ESP32 UART Driver</t>
         </is>
       </c>
       <c r="E64" s="14" t="inlineStr">
         <is>
-          <t>Simulate ESP32 optical triggers and servo responses in unit tests</t>
+          <t>Thread 3: Non-blocking serial worker communicating at 115200 baud</t>
         </is>
       </c>
       <c r="F64" s="14" t="inlineStr">
         <is>
-          <t>AGENTS.md Firmware</t>
+          <t>System Flowchart Node 17</t>
         </is>
       </c>
       <c r="G64" s="13" t="inlineStr">
@@ -4099,7 +4092,7 @@
       </c>
       <c r="I64" s="13" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J64" s="14" t="inlineStr">
@@ -4111,7 +4104,7 @@
     <row r="65" ht="22" customHeight="1">
       <c r="A65" s="16" t="inlineStr">
         <is>
-          <t>TASK-EDGE-TRK-01</t>
+          <t>TASK-EDGE-SER-02</t>
         </is>
       </c>
       <c r="B65" s="16" t="inlineStr">
@@ -4126,17 +4119,17 @@
       </c>
       <c r="D65" s="17" t="inlineStr">
         <is>
-          <t>Cradle Tracking FIFO Queue</t>
+          <t>Serial Mock Driver for Hardware-Free Dev</t>
         </is>
       </c>
       <c r="E65" s="17" t="inlineStr">
         <is>
-          <t>Maintain cradle queue mapping cradle_id from image station to sorting gate</t>
+          <t>Simulate ESP32 optical triggers and servo responses in unit tests</t>
         </is>
       </c>
       <c r="F65" s="17" t="inlineStr">
         <is>
-          <t>System Flowchart Node 5,11</t>
+          <t>AGENTS.md Firmware</t>
         </is>
       </c>
       <c r="G65" s="16" t="inlineStr">
@@ -4144,26 +4137,26 @@
           <t>Codex</t>
         </is>
       </c>
-      <c r="H65" s="18" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="H65" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I65" s="16" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J65" s="17" t="inlineStr">
         <is>
-          <t>test_cradle_tracking_queue.py</t>
+          <t>test_esp32_serial_mock_and_motor_commands</t>
         </is>
       </c>
     </row>
     <row r="66" ht="22" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>TASK-EDGE-TRK-02</t>
+          <t>TASK-EDGE-TRK-01</t>
         </is>
       </c>
       <c r="B66" s="13" t="inlineStr">
@@ -4178,17 +4171,17 @@
       </c>
       <c r="D66" s="14" t="inlineStr">
         <is>
-          <t>Conveyor Index Resynchronization Handler</t>
+          <t>Cradle Tracking FIFO Queue</t>
         </is>
       </c>
       <c r="E66" s="14" t="inlineStr">
         <is>
-          <t>Pause conveyor and alert operator if physical cradle index drifts</t>
+          <t>Maintain cradle queue mapping cradle_id from image station to sorting gate</t>
         </is>
       </c>
       <c r="F66" s="14" t="inlineStr">
         <is>
-          <t>System Flowchart Node 15,16</t>
+          <t>System Flowchart Node 5,11</t>
         </is>
       </c>
       <c r="G66" s="13" t="inlineStr">
@@ -4203,19 +4196,19 @@
       </c>
       <c r="I66" s="13" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J66" s="14" t="inlineStr">
         <is>
-          <t>test_cradle_resync_handler.py</t>
+          <t>test_cradle_tracking_queue.py</t>
         </is>
       </c>
     </row>
     <row r="67" ht="22" customHeight="1">
       <c r="A67" s="16" t="inlineStr">
         <is>
-          <t>TASK-EDGE-REV-01</t>
+          <t>TASK-EDGE-TRK-02</t>
         </is>
       </c>
       <c r="B67" s="16" t="inlineStr">
@@ -4230,17 +4223,17 @@
       </c>
       <c r="D67" s="17" t="inlineStr">
         <is>
-          <t>Manual Review Fallback State Machine</t>
+          <t>Conveyor Index Resynchronization Handler</t>
         </is>
       </c>
       <c r="E67" s="17" t="inlineStr">
         <is>
-          <t>Trigger manual review flag when confidence &lt; 0.75 or egg uncentered</t>
+          <t>Pause conveyor and alert operator if physical cradle index drifts</t>
         </is>
       </c>
       <c r="F67" s="17" t="inlineStr">
         <is>
-          <t>System Flowchart Node 9,10</t>
+          <t>System Flowchart Node 15,16</t>
         </is>
       </c>
       <c r="G67" s="16" t="inlineStr">
@@ -4255,19 +4248,19 @@
       </c>
       <c r="I67" s="16" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J67" s="17" t="inlineStr">
         <is>
-          <t>test_manual_review_fallback.py</t>
+          <t>test_cradle_resync_handler.py</t>
         </is>
       </c>
     </row>
     <row r="68" ht="22" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>TASK-EDGE-UI-01</t>
+          <t>TASK-EDGE-REV-01</t>
         </is>
       </c>
       <c r="B68" s="13" t="inlineStr">
@@ -4282,17 +4275,17 @@
       </c>
       <c r="D68" s="14" t="inlineStr">
         <is>
-          <t>CustomTkinter 60 FPS Operator Desktop UI</t>
+          <t>Manual Review Fallback State Machine</t>
         </is>
       </c>
       <c r="E68" s="14" t="inlineStr">
         <is>
-          <t>Main Thread: CustomTkinter operator GUI with Foundation University theme</t>
+          <t>Trigger manual review flag when confidence &lt; 0.75 or egg uncentered</t>
         </is>
       </c>
       <c r="F68" s="14" t="inlineStr">
         <is>
-          <t>Use Case: Worker</t>
+          <t>System Flowchart Node 9,10</t>
         </is>
       </c>
       <c r="G68" s="13" t="inlineStr">
@@ -4300,9 +4293,9 @@
           <t>Codex</t>
         </is>
       </c>
-      <c r="H68" s="15" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="H68" s="18" t="inlineStr">
+        <is>
+          <t>Backlog</t>
         </is>
       </c>
       <c r="I68" s="13" t="inlineStr">
@@ -4312,14 +4305,14 @@
       </c>
       <c r="J68" s="14" t="inlineStr">
         <is>
-          <t>Desktop UI smoke launch</t>
+          <t>test_manual_review_fallback.py</t>
         </is>
       </c>
     </row>
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="16" t="inlineStr">
         <is>
-          <t>TASK-EDGE-UI-02</t>
+          <t>TASK-EDGE-UI-01</t>
         </is>
       </c>
       <c r="B69" s="16" t="inlineStr">
@@ -4334,12 +4327,12 @@
       </c>
       <c r="D69" s="17" t="inlineStr">
         <is>
-          <t>Live Candling Video Viewport</t>
+          <t>CustomTkinter 60 FPS Operator Desktop UI</t>
         </is>
       </c>
       <c r="E69" s="17" t="inlineStr">
         <is>
-          <t>Smooth video rendering canvas with overlay bounding box and class tag</t>
+          <t>Main Thread: CustomTkinter operator GUI with Foundation University theme</t>
         </is>
       </c>
       <c r="F69" s="17" t="inlineStr">
@@ -4364,14 +4357,14 @@
       </c>
       <c r="J69" s="17" t="inlineStr">
         <is>
-          <t>Desktop UI verification</t>
+          <t>Desktop UI smoke launch</t>
         </is>
       </c>
     </row>
     <row r="70" ht="22" customHeight="1">
       <c r="A70" s="13" t="inlineStr">
         <is>
-          <t>TASK-EDGE-UI-03</t>
+          <t>TASK-EDGE-UI-02</t>
         </is>
       </c>
       <c r="B70" s="13" t="inlineStr">
@@ -4386,12 +4379,12 @@
       </c>
       <c r="D70" s="14" t="inlineStr">
         <is>
-          <t>Real-Time Session Statistics Counters</t>
+          <t>Live Candling Video Viewport</t>
         </is>
       </c>
       <c r="E70" s="14" t="inlineStr">
         <is>
-          <t>Live counters for Fertile, Infertile, and Manual Review count</t>
+          <t>Smooth video rendering canvas with overlay bounding box and class tag</t>
         </is>
       </c>
       <c r="F70" s="14" t="inlineStr">
@@ -4411,7 +4404,7 @@
       </c>
       <c r="I70" s="13" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J70" s="14" t="inlineStr">
@@ -4423,7 +4416,7 @@
     <row r="71" ht="22" customHeight="1">
       <c r="A71" s="16" t="inlineStr">
         <is>
-          <t>TASK-EDGE-UI-04</t>
+          <t>TASK-EDGE-UI-03</t>
         </is>
       </c>
       <c r="B71" s="16" t="inlineStr">
@@ -4438,17 +4431,17 @@
       </c>
       <c r="D71" s="17" t="inlineStr">
         <is>
-          <t>Interactive Manual Override Dialog Modal</t>
+          <t>Real-Time Session Statistics Counters</t>
         </is>
       </c>
       <c r="E71" s="17" t="inlineStr">
         <is>
-          <t>Modal popup enabling operator to inspect flagged egg and confirm class</t>
+          <t>Live counters for Fertile, Infertile, and Manual Review</t>
         </is>
       </c>
       <c r="F71" s="17" t="inlineStr">
         <is>
-          <t>System Flowchart Node 10</t>
+          <t>Use Case: Worker</t>
         </is>
       </c>
       <c r="G71" s="16" t="inlineStr">
@@ -4456,26 +4449,26 @@
           <t>Codex</t>
         </is>
       </c>
-      <c r="H71" s="18" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="H71" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I71" s="16" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J71" s="17" t="inlineStr">
         <is>
-          <t>Desktop UI modal test</t>
+          <t>Desktop UI verification</t>
         </is>
       </c>
     </row>
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="13" t="inlineStr">
         <is>
-          <t>TASK-EDGE-UI-05</t>
+          <t>TASK-EDGE-UI-04</t>
         </is>
       </c>
       <c r="B72" s="13" t="inlineStr">
@@ -4490,17 +4483,17 @@
       </c>
       <c r="D72" s="14" t="inlineStr">
         <is>
-          <t>Conveyor Pause &amp; Emergency Stop Controls</t>
+          <t>Interactive Manual Override Dialog Modal</t>
         </is>
       </c>
       <c r="E72" s="14" t="inlineStr">
         <is>
-          <t>Instant physical rig pause and serial E-STOP command dispatch</t>
+          <t>Modal popup enabling operator to inspect flagged egg and confirm class</t>
         </is>
       </c>
       <c r="F72" s="14" t="inlineStr">
         <is>
-          <t>System Flowchart Node 16</t>
+          <t>System Flowchart Node 10</t>
         </is>
       </c>
       <c r="G72" s="13" t="inlineStr">
@@ -4508,51 +4501,51 @@
           <t>Codex</t>
         </is>
       </c>
-      <c r="H72" s="15" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="H72" s="18" t="inlineStr">
+        <is>
+          <t>Backlog</t>
         </is>
       </c>
       <c r="I72" s="13" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J72" s="14" t="inlineStr">
         <is>
-          <t>Desktop UI verification</t>
+          <t>Desktop UI modal test</t>
         </is>
       </c>
     </row>
     <row r="73" ht="22" customHeight="1">
       <c r="A73" s="16" t="inlineStr">
         <is>
-          <t>TASK-DASH-PG-01</t>
+          <t>TASK-EDGE-UI-05</t>
         </is>
       </c>
       <c r="B73" s="16" t="inlineStr">
         <is>
-          <t>Phase 4D: Dashboard</t>
+          <t>Phase 4B: Edge App</t>
         </is>
       </c>
       <c r="C73" s="17" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Edge CV</t>
         </is>
       </c>
       <c r="D73" s="17" t="inlineStr">
         <is>
-          <t>LoginPage.tsx with JWT Auth</t>
+          <t>Conveyor Pause &amp; Emergency Stop Controls</t>
         </is>
       </c>
       <c r="E73" s="17" t="inlineStr">
         <is>
-          <t>Login view with Foundation University maroon branding and token persistence</t>
+          <t>Instant physical rig pause and serial E-STOP command dispatch</t>
         </is>
       </c>
       <c r="F73" s="17" t="inlineStr">
         <is>
-          <t>Use Case: Worker</t>
+          <t>System Flowchart Node 16</t>
         </is>
       </c>
       <c r="G73" s="16" t="inlineStr">
@@ -4567,19 +4560,19 @@
       </c>
       <c r="I73" s="16" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J73" s="17" t="inlineStr">
         <is>
-          <t>npm.cmd run build</t>
+          <t>Desktop UI verification</t>
         </is>
       </c>
     </row>
     <row r="74" ht="22" customHeight="1">
       <c r="A74" s="13" t="inlineStr">
         <is>
-          <t>TASK-DASH-PG-02</t>
+          <t>TASK-DASH-PG-01</t>
         </is>
       </c>
       <c r="B74" s="13" t="inlineStr">
@@ -4594,17 +4587,17 @@
       </c>
       <c r="D74" s="14" t="inlineStr">
         <is>
-          <t>OverviewPage.tsx Real-Time KPI Cards</t>
+          <t>LoginPage.tsx with JWT Auth</t>
         </is>
       </c>
       <c r="E74" s="14" t="inlineStr">
         <is>
-          <t>High-level summary of active batches, fertility %, and today's sorting volume</t>
+          <t>Login view with Foundation University maroon branding and token persistence</t>
         </is>
       </c>
       <c r="F74" s="14" t="inlineStr">
         <is>
-          <t>Use Case: Supervisor</t>
+          <t>Use Case: Worker</t>
         </is>
       </c>
       <c r="G74" s="13" t="inlineStr">
@@ -4631,7 +4624,7 @@
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="16" t="inlineStr">
         <is>
-          <t>TASK-DASH-PG-03</t>
+          <t>TASK-DASH-PG-02</t>
         </is>
       </c>
       <c r="B75" s="16" t="inlineStr">
@@ -4646,12 +4639,12 @@
       </c>
       <c r="D75" s="17" t="inlineStr">
         <is>
-          <t>BatchesPage.tsx Lifecycle Management</t>
+          <t>OverviewPage.tsx Real-Time KPI Cards</t>
         </is>
       </c>
       <c r="E75" s="17" t="inlineStr">
         <is>
-          <t>Table of all batches, stage advancement modal (Day 10, Hatched, Completed), hatch closure</t>
+          <t>High-level summary of active batches, fertility %, and today's sorting volume</t>
         </is>
       </c>
       <c r="F75" s="17" t="inlineStr">
@@ -4683,7 +4676,7 @@
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="13" t="inlineStr">
         <is>
-          <t>TASK-DASH-PG-04</t>
+          <t>TASK-DASH-PG-03</t>
         </is>
       </c>
       <c r="B76" s="13" t="inlineStr">
@@ -4698,12 +4691,12 @@
       </c>
       <c r="D76" s="14" t="inlineStr">
         <is>
-          <t>ScanExplorerPage.tsx Visual Search</t>
+          <t>BatchesPage.tsx Lifecycle Management</t>
         </is>
       </c>
       <c r="E76" s="14" t="inlineStr">
         <is>
-          <t>Filterable grid of historical scan captures with image lightbox inspection</t>
+          <t>Table of all batches, Day 10 stage advancement, and hatch closure</t>
         </is>
       </c>
       <c r="F76" s="14" t="inlineStr">
@@ -4723,7 +4716,7 @@
       </c>
       <c r="I76" s="13" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J76" s="14" t="inlineStr">
@@ -4735,7 +4728,7 @@
     <row r="77" ht="22" customHeight="1">
       <c r="A77" s="16" t="inlineStr">
         <is>
-          <t>TASK-DASH-PG-05</t>
+          <t>TASK-DASH-PG-04</t>
         </is>
       </c>
       <c r="B77" s="16" t="inlineStr">
@@ -4750,12 +4743,12 @@
       </c>
       <c r="D77" s="17" t="inlineStr">
         <is>
-          <t>AnalyticsPage.tsx Multi-Chart Suite</t>
+          <t>ScanExplorerPage.tsx Visual Search</t>
         </is>
       </c>
       <c r="E77" s="17" t="inlineStr">
         <is>
-          <t>Recharts visualizer for mortality curves, breed comparisons, and Penoy revenue</t>
+          <t>Filterable grid of historical scan captures with image lightbox inspection</t>
         </is>
       </c>
       <c r="F77" s="17" t="inlineStr">
@@ -4775,7 +4768,7 @@
       </c>
       <c r="I77" s="16" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J77" s="17" t="inlineStr">
@@ -4787,7 +4780,7 @@
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="13" t="inlineStr">
         <is>
-          <t>TASK-DASH-PG-06</t>
+          <t>TASK-DASH-PG-05</t>
         </is>
       </c>
       <c r="B78" s="13" t="inlineStr">
@@ -4802,12 +4795,12 @@
       </c>
       <c r="D78" s="14" t="inlineStr">
         <is>
-          <t>RecordsPage.tsx Audit Archive</t>
+          <t>AnalyticsPage.tsx Multi-Chart Suite</t>
         </is>
       </c>
       <c r="E78" s="14" t="inlineStr">
         <is>
-          <t>Historical scan and session records table with one-click CSV/PDF download</t>
+          <t>Recharts visualizer for mortality curves, breed comparisons, and Penoy revenue</t>
         </is>
       </c>
       <c r="F78" s="14" t="inlineStr">
@@ -4827,7 +4820,7 @@
       </c>
       <c r="I78" s="13" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J78" s="14" t="inlineStr">
@@ -4839,7 +4832,7 @@
     <row r="79" ht="22" customHeight="1">
       <c r="A79" s="16" t="inlineStr">
         <is>
-          <t>TASK-DASH-PG-07</t>
+          <t>TASK-DASH-PG-06</t>
         </is>
       </c>
       <c r="B79" s="16" t="inlineStr">
@@ -4854,17 +4847,17 @@
       </c>
       <c r="D79" s="17" t="inlineStr">
         <is>
-          <t>DevicesPage.tsx Hardware Monitor</t>
+          <t>RecordsPage.tsx Audit Archive</t>
         </is>
       </c>
       <c r="E79" s="17" t="inlineStr">
         <is>
-          <t>Live cards showing connected Raspberry Pi and ESP32 sorter rigs</t>
+          <t>Historical scan and session records table with one-click CSV/PDF download</t>
         </is>
       </c>
       <c r="F79" s="17" t="inlineStr">
         <is>
-          <t>Use Case: Admin</t>
+          <t>Use Case: Supervisor</t>
         </is>
       </c>
       <c r="G79" s="16" t="inlineStr">
@@ -4891,7 +4884,7 @@
     <row r="80" ht="22" customHeight="1">
       <c r="A80" s="13" t="inlineStr">
         <is>
-          <t>TASK-DASH-PG-08</t>
+          <t>TASK-DASH-PG-07</t>
         </is>
       </c>
       <c r="B80" s="13" t="inlineStr">
@@ -4906,12 +4899,12 @@
       </c>
       <c r="D80" s="14" t="inlineStr">
         <is>
-          <t>ModelsPage.tsx MLOps Registry</t>
+          <t>DevicesPage.tsx Hardware Monitor</t>
         </is>
       </c>
       <c r="E80" s="14" t="inlineStr">
         <is>
-          <t>View deployed YOLOv8 ONNX model version, latency benchmarks, thresholds</t>
+          <t>Live cards showing connected Raspberry Pi and ESP32 sorter rigs</t>
         </is>
       </c>
       <c r="F80" s="14" t="inlineStr">
@@ -4943,7 +4936,7 @@
     <row r="81" ht="22" customHeight="1">
       <c r="A81" s="16" t="inlineStr">
         <is>
-          <t>TASK-DASH-PG-09</t>
+          <t>TASK-DASH-PG-08</t>
         </is>
       </c>
       <c r="B81" s="16" t="inlineStr">
@@ -4958,12 +4951,12 @@
       </c>
       <c r="D81" s="17" t="inlineStr">
         <is>
-          <t>UsersPage.tsx User Administration</t>
+          <t>ModelsPage.tsx MLOps Registry</t>
         </is>
       </c>
       <c r="E81" s="17" t="inlineStr">
         <is>
-          <t>Admin table for managing operator, supervisor, and administrator accounts</t>
+          <t>View deployed YOLOv8 ONNX model version, latency benchmarks, thresholds</t>
         </is>
       </c>
       <c r="F81" s="17" t="inlineStr">
@@ -4983,7 +4976,7 @@
       </c>
       <c r="I81" s="16" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J81" s="17" t="inlineStr">
@@ -4995,7 +4988,7 @@
     <row r="82" ht="22" customHeight="1">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>TASK-DASH-PG-10</t>
+          <t>TASK-DASH-PG-09</t>
         </is>
       </c>
       <c r="B82" s="13" t="inlineStr">
@@ -5010,12 +5003,12 @@
       </c>
       <c r="D82" s="14" t="inlineStr">
         <is>
-          <t>AuditLogsPage.tsx Security Trail</t>
+          <t>UsersPage.tsx User Administration</t>
         </is>
       </c>
       <c r="E82" s="14" t="inlineStr">
         <is>
-          <t>Chronological table of all system events, login attempts, and overrides</t>
+          <t>Admin table for managing operator, supervisor, and administrator accounts</t>
         </is>
       </c>
       <c r="F82" s="14" t="inlineStr">
@@ -5047,7 +5040,7 @@
     <row r="83" ht="22" customHeight="1">
       <c r="A83" s="16" t="inlineStr">
         <is>
-          <t>TASK-DASH-PG-11</t>
+          <t>TASK-DASH-PG-10</t>
         </is>
       </c>
       <c r="B83" s="16" t="inlineStr">
@@ -5062,12 +5055,12 @@
       </c>
       <c r="D83" s="17" t="inlineStr">
         <is>
-          <t>SettingsPage.tsx System Configuration</t>
+          <t>AuditLogsPage.tsx Security Trail</t>
         </is>
       </c>
       <c r="E83" s="17" t="inlineStr">
         <is>
-          <t>Configure Penoy price (P14), confidence thresholds, and DB backup downloads</t>
+          <t>Chronological table of all system events, login attempts, and overrides</t>
         </is>
       </c>
       <c r="F83" s="17" t="inlineStr">
@@ -5087,7 +5080,7 @@
       </c>
       <c r="I83" s="16" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J83" s="17" t="inlineStr">
@@ -5099,7 +5092,7 @@
     <row r="84" ht="22" customHeight="1">
       <c r="A84" s="13" t="inlineStr">
         <is>
-          <t>TASK-DASH-CP-01</t>
+          <t>TASK-DASH-PG-11</t>
         </is>
       </c>
       <c r="B84" s="13" t="inlineStr">
@@ -5114,17 +5107,17 @@
       </c>
       <c r="D84" s="14" t="inlineStr">
         <is>
-          <t>Incubation Tray Matrix (42 Slots A1-F7)</t>
+          <t>SettingsPage.tsx System Configuration</t>
         </is>
       </c>
       <c r="E84" s="14" t="inlineStr">
         <is>
-          <t>Interactive SVG grid showing physical incubator tray slot occupancy and status</t>
+          <t>Configure Penoy price (P14), confidence thresholds, and DB backup downloads</t>
         </is>
       </c>
       <c r="F84" s="14" t="inlineStr">
         <is>
-          <t>Use Case: Supervisor</t>
+          <t>Use Case: Admin</t>
         </is>
       </c>
       <c r="G84" s="13" t="inlineStr">
@@ -5139,7 +5132,7 @@
       </c>
       <c r="I84" s="13" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J84" s="14" t="inlineStr">
@@ -5151,7 +5144,7 @@
     <row r="85" ht="22" customHeight="1">
       <c r="A85" s="16" t="inlineStr">
         <is>
-          <t>TASK-DASH-CP-02</t>
+          <t>TASK-DASH-CP-01</t>
         </is>
       </c>
       <c r="B85" s="16" t="inlineStr">
@@ -5166,17 +5159,17 @@
       </c>
       <c r="D85" s="17" t="inlineStr">
         <is>
-          <t>Interactive Penoy Economic Calculator</t>
+          <t>Incubation Tray Matrix (42 Slots A1-F7)</t>
         </is>
       </c>
       <c r="E85" s="17" t="inlineStr">
         <is>
-          <t>Widget computing Day 10 salvage income based on P14.00/egg price</t>
+          <t>Interactive SVG grid showing physical incubator tray slot occupancy and status</t>
         </is>
       </c>
       <c r="F85" s="17" t="inlineStr">
         <is>
-          <t>AGENTS.md Tenet 3</t>
+          <t>Use Case: Supervisor</t>
         </is>
       </c>
       <c r="G85" s="16" t="inlineStr">
@@ -5191,7 +5184,7 @@
       </c>
       <c r="I85" s="16" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J85" s="17" t="inlineStr">
@@ -5203,7 +5196,7 @@
     <row r="86" ht="22" customHeight="1">
       <c r="A86" s="13" t="inlineStr">
         <is>
-          <t>TASK-DASH-CP-03</t>
+          <t>TASK-DASH-CP-02</t>
         </is>
       </c>
       <c r="B86" s="13" t="inlineStr">
@@ -5218,17 +5211,17 @@
       </c>
       <c r="D86" s="14" t="inlineStr">
         <is>
-          <t>Breed Filter: IP-Itim, Khaki, Kayumanggi</t>
+          <t>Interactive Penoy Economic Calculator</t>
         </is>
       </c>
       <c r="E86" s="14" t="inlineStr">
         <is>
-          <t>Dropdown to isolate metrics by pure line vs commercial hybrid</t>
+          <t>Widget computing Day 10 salvage income based on P14.00/egg price</t>
         </is>
       </c>
       <c r="F86" s="14" t="inlineStr">
         <is>
-          <t>Methodology 3.1</t>
+          <t>AGENTS.md Tenet 3</t>
         </is>
       </c>
       <c r="G86" s="13" t="inlineStr">
@@ -5255,7 +5248,7 @@
     <row r="87" ht="22" customHeight="1">
       <c r="A87" s="16" t="inlineStr">
         <is>
-          <t>TASK-DASH-CP-04</t>
+          <t>TASK-DASH-CP-03</t>
         </is>
       </c>
       <c r="B87" s="16" t="inlineStr">
@@ -5270,12 +5263,12 @@
       </c>
       <c r="D87" s="17" t="inlineStr">
         <is>
-          <t>Stage Filter: Setting, Day 10, Hatched, Completed</t>
+          <t>Breed Filter: IP-Itim, Khaki, Kayumanggi</t>
         </is>
       </c>
       <c r="E87" s="17" t="inlineStr">
         <is>
-          <t>Toggle to filter analysis by incubation stage milestone</t>
+          <t>Dropdown to isolate metrics by pure line vs commercial hybrid</t>
         </is>
       </c>
       <c r="F87" s="17" t="inlineStr">
@@ -5307,7 +5300,7 @@
     <row r="88" ht="22" customHeight="1">
       <c r="A88" s="13" t="inlineStr">
         <is>
-          <t>TASK-DASH-CP-05</t>
+          <t>TASK-DASH-CP-04</t>
         </is>
       </c>
       <c r="B88" s="13" t="inlineStr">
@@ -5322,17 +5315,17 @@
       </c>
       <c r="D88" s="14" t="inlineStr">
         <is>
-          <t>Dark / Light Mode Theme System</t>
+          <t>Day 10 Filter</t>
         </is>
       </c>
       <c r="E88" s="14" t="inlineStr">
         <is>
-          <t>TailwindCSS theme switcher with FU Maroon (#800000) accents</t>
+          <t>Filter analytics for the single Day 10 checkpoint</t>
         </is>
       </c>
       <c r="F88" s="14" t="inlineStr">
         <is>
-          <t>AGENTS.md FU Brand</t>
+          <t>Methodology 3.1</t>
         </is>
       </c>
       <c r="G88" s="13" t="inlineStr">
@@ -5347,7 +5340,7 @@
       </c>
       <c r="I88" s="13" t="inlineStr">
         <is>
-          <t>P2 - Medium</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J88" s="14" t="inlineStr">
@@ -5359,32 +5352,32 @@
     <row r="89" ht="22" customHeight="1">
       <c r="A89" s="16" t="inlineStr">
         <is>
-          <t>TASK-FW-INT-01</t>
+          <t>TASK-DASH-CP-05</t>
         </is>
       </c>
       <c r="B89" s="16" t="inlineStr">
         <is>
-          <t>Phase 4A: Firmware</t>
+          <t>Phase 4D: Dashboard</t>
         </is>
       </c>
       <c r="C89" s="17" t="inlineStr">
         <is>
-          <t>Firmware</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D89" s="17" t="inlineStr">
         <is>
-          <t>Optical Sensor Hardware Interrupt</t>
+          <t>Dark / Light Mode Theme System</t>
         </is>
       </c>
       <c r="E89" s="17" t="inlineStr">
         <is>
-          <t>ESP32 GPIO 14 optical beam-break edge detection interrupt</t>
+          <t>TailwindCSS theme switcher with FU Maroon (#800000) accents</t>
         </is>
       </c>
       <c r="F89" s="17" t="inlineStr">
         <is>
-          <t>System Flowchart</t>
+          <t>AGENTS.md FU Brand</t>
         </is>
       </c>
       <c r="G89" s="16" t="inlineStr">
@@ -5399,19 +5392,19 @@
       </c>
       <c r="I89" s="16" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P2 - Medium</t>
         </is>
       </c>
       <c r="J89" s="17" t="inlineStr">
         <is>
-          <t>esp32_actuator.ino review</t>
+          <t>npm.cmd run build</t>
         </is>
       </c>
     </row>
     <row r="90" ht="22" customHeight="1">
       <c r="A90" s="13" t="inlineStr">
         <is>
-          <t>TASK-FW-INT-02</t>
+          <t>TASK-FW-INT-01</t>
         </is>
       </c>
       <c r="B90" s="13" t="inlineStr">
@@ -5426,17 +5419,17 @@
       </c>
       <c r="D90" s="14" t="inlineStr">
         <is>
-          <t>600ms Hardware Optical Debounce Lockout</t>
+          <t>Optical Sensor Hardware Interrupt</t>
         </is>
       </c>
       <c r="E90" s="14" t="inlineStr">
         <is>
-          <t>Non-blocking timer lockout preventing false double-triggers on single egg</t>
+          <t>ESP32 GPIO 14 optical beam-break edge detection interrupt</t>
         </is>
       </c>
       <c r="F90" s="14" t="inlineStr">
         <is>
-          <t>AGENTS.md Firmware</t>
+          <t>System Flowchart</t>
         </is>
       </c>
       <c r="G90" s="13" t="inlineStr">
@@ -5463,7 +5456,7 @@
     <row r="91" ht="22" customHeight="1">
       <c r="A91" s="16" t="inlineStr">
         <is>
-          <t>TASK-FW-LED-01</t>
+          <t>TASK-FW-INT-02</t>
         </is>
       </c>
       <c r="B91" s="16" t="inlineStr">
@@ -5478,17 +5471,17 @@
       </c>
       <c r="D91" s="17" t="inlineStr">
         <is>
-          <t>Candling Strobe LED Driver Relay</t>
+          <t>600ms Hardware Optical Debounce Lockout</t>
         </is>
       </c>
       <c r="E91" s="17" t="inlineStr">
         <is>
-          <t>GPIO 19 strobe trigger synchronized with camera exposure</t>
+          <t>Non-blocking timer lockout preventing false double-triggers on single egg</t>
         </is>
       </c>
       <c r="F91" s="17" t="inlineStr">
         <is>
-          <t>System Flowchart Node 7</t>
+          <t>AGENTS.md Firmware</t>
         </is>
       </c>
       <c r="G91" s="16" t="inlineStr">
@@ -5503,7 +5496,7 @@
       </c>
       <c r="I91" s="16" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J91" s="17" t="inlineStr">
@@ -5515,7 +5508,7 @@
     <row r="92" ht="22" customHeight="1">
       <c r="A92" s="13" t="inlineStr">
         <is>
-          <t>TASK-FW-SER-01</t>
+          <t>TASK-FW-LED-01</t>
         </is>
       </c>
       <c r="B92" s="13" t="inlineStr">
@@ -5530,17 +5523,17 @@
       </c>
       <c r="D92" s="14" t="inlineStr">
         <is>
-          <t>Non-Blocking Serial UART Command Parser</t>
+          <t>Candling Strobe LED Driver Relay</t>
         </is>
       </c>
       <c r="E92" s="14" t="inlineStr">
         <is>
-          <t>Buffer incoming 115200 baud UART bytes without delay() calls</t>
+          <t>GPIO 19 strobe trigger synchronized with camera exposure</t>
         </is>
       </c>
       <c r="F92" s="14" t="inlineStr">
         <is>
-          <t>AGENTS.md Firmware</t>
+          <t>System Flowchart Node 7</t>
         </is>
       </c>
       <c r="G92" s="13" t="inlineStr">
@@ -5555,7 +5548,7 @@
       </c>
       <c r="I92" s="13" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J92" s="14" t="inlineStr">
@@ -5567,7 +5560,7 @@
     <row r="93" ht="22" customHeight="1">
       <c r="A93" s="16" t="inlineStr">
         <is>
-          <t>TASK-FW-SER-02</t>
+          <t>TASK-FW-SER-01</t>
         </is>
       </c>
       <c r="B93" s="16" t="inlineStr">
@@ -5582,17 +5575,17 @@
       </c>
       <c r="D93" s="17" t="inlineStr">
         <is>
-          <t>Serial ACK / NACK Status Protocol</t>
+          <t>Non-Blocking Serial UART Command Parser</t>
         </is>
       </c>
       <c r="E93" s="17" t="inlineStr">
         <is>
-          <t>Transmit acknowledgement packets upon command execution to edge driver</t>
+          <t>Buffer incoming 115200 baud UART bytes without delay() calls</t>
         </is>
       </c>
       <c r="F93" s="17" t="inlineStr">
         <is>
-          <t>System Flowchart Node 3</t>
+          <t>AGENTS.md Firmware</t>
         </is>
       </c>
       <c r="G93" s="16" t="inlineStr">
@@ -5607,7 +5600,7 @@
       </c>
       <c r="I93" s="16" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J93" s="17" t="inlineStr">
@@ -5619,7 +5612,7 @@
     <row r="94" ht="22" customHeight="1">
       <c r="A94" s="13" t="inlineStr">
         <is>
-          <t>TASK-FW-STP-01</t>
+          <t>TASK-FW-SER-02</t>
         </is>
       </c>
       <c r="B94" s="13" t="inlineStr">
@@ -5634,17 +5627,17 @@
       </c>
       <c r="D94" s="14" t="inlineStr">
         <is>
-          <t>Stepper Pocket-Conveyor Transport Routine</t>
+          <t>Serial ACK / NACK Status Protocol</t>
         </is>
       </c>
       <c r="E94" s="14" t="inlineStr">
         <is>
-          <t>Indexed step timing to advance pocket conveyor one cradle at a time</t>
+          <t>Transmit acknowledgement packets upon command execution to edge driver</t>
         </is>
       </c>
       <c r="F94" s="14" t="inlineStr">
         <is>
-          <t>System Flowchart Node 6,14</t>
+          <t>System Flowchart Node 3</t>
         </is>
       </c>
       <c r="G94" s="13" t="inlineStr">
@@ -5659,19 +5652,19 @@
       </c>
       <c r="I94" s="13" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J94" s="14" t="inlineStr">
         <is>
-          <t>Firmware bench test</t>
+          <t>Serial loopback test</t>
         </is>
       </c>
     </row>
     <row r="95" ht="22" customHeight="1">
       <c r="A95" s="16" t="inlineStr">
         <is>
-          <t>TASK-FW-SRV-01</t>
+          <t>TASK-FW-STP-01</t>
         </is>
       </c>
       <c r="B95" s="16" t="inlineStr">
@@ -5686,17 +5679,17 @@
       </c>
       <c r="D95" s="17" t="inlineStr">
         <is>
-          <t>Servo Diverter (Fertile Pass-Through)</t>
+          <t>Stepper Pocket-Conveyor Transport Routine</t>
         </is>
       </c>
       <c r="E95" s="17" t="inlineStr">
         <is>
-          <t>Maintain idle servo position (0 deg) allowing Fertile eggs to continue to incubation tray</t>
+          <t>Indexed step timing to advance pocket conveyor one cradle at a time</t>
         </is>
       </c>
       <c r="F95" s="17" t="inlineStr">
         <is>
-          <t>System Flowchart Node 18</t>
+          <t>System Flowchart Node 6,14</t>
         </is>
       </c>
       <c r="G95" s="16" t="inlineStr">
@@ -5704,9 +5697,9 @@
           <t>Codex</t>
         </is>
       </c>
-      <c r="H95" s="15" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="H95" s="18" t="inlineStr">
+        <is>
+          <t>Backlog</t>
         </is>
       </c>
       <c r="I95" s="16" t="inlineStr">
@@ -5716,14 +5709,14 @@
       </c>
       <c r="J95" s="17" t="inlineStr">
         <is>
-          <t>esp32_actuator.ino review</t>
+          <t>Firmware bench test</t>
         </is>
       </c>
     </row>
     <row r="96" ht="22" customHeight="1">
       <c r="A96" s="13" t="inlineStr">
         <is>
-          <t>TASK-FW-SRV-02</t>
+          <t>TASK-FW-SRV-01</t>
         </is>
       </c>
       <c r="B96" s="13" t="inlineStr">
@@ -5738,17 +5731,17 @@
       </c>
       <c r="D96" s="14" t="inlineStr">
         <is>
-          <t>Servo Diverter (Infertile / Penoy Salvage)</t>
+          <t>Servo Gate 1 (Fertile Release)</t>
         </is>
       </c>
       <c r="E96" s="14" t="inlineStr">
         <is>
-          <t>Actuate servo diverter (60 deg) for Day 10 Penoy salvage sale (@ P14.00)</t>
+          <t>Actuate servo diverter for Fertile eggs into cushioned incubation tray</t>
         </is>
       </c>
       <c r="F96" s="14" t="inlineStr">
         <is>
-          <t>System Flowchart Node 19</t>
+          <t>System Flowchart Node 18</t>
         </is>
       </c>
       <c r="G96" s="13" t="inlineStr">
@@ -5775,7 +5768,7 @@
     <row r="97" ht="22" customHeight="1">
       <c r="A97" s="16" t="inlineStr">
         <is>
-          <t>TASK-FW-KIN-01</t>
+          <t>TASK-FW-SRV-02</t>
         </is>
       </c>
       <c r="B97" s="16" t="inlineStr">
@@ -5790,17 +5783,17 @@
       </c>
       <c r="D97" s="17" t="inlineStr">
         <is>
-          <t>Kinematic Actuation Delay Timer</t>
+          <t>Servo Gate 2 (Infertile / Penoy Salvage)</t>
         </is>
       </c>
       <c r="E97" s="17" t="inlineStr">
         <is>
-          <t>Calculate Delta-t = D / v = 25cm / 12.5cm/s = 2000ms delay before servo firing</t>
+          <t>Actuate servo diverter for Day 10 Penoy salvage sale (@ P14.00)</t>
         </is>
       </c>
       <c r="F97" s="17" t="inlineStr">
         <is>
-          <t>Methodology 3.4</t>
+          <t>System Flowchart Node 19</t>
         </is>
       </c>
       <c r="G97" s="16" t="inlineStr">
@@ -5808,9 +5801,9 @@
           <t>Codex</t>
         </is>
       </c>
-      <c r="H97" s="15" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="H97" s="18" t="inlineStr">
+        <is>
+          <t>Backlog</t>
         </is>
       </c>
       <c r="I97" s="16" t="inlineStr">
@@ -5820,39 +5813,39 @@
       </c>
       <c r="J97" s="17" t="inlineStr">
         <is>
-          <t>esp32_actuator.ino review</t>
+          <t>Firmware bench test</t>
         </is>
       </c>
     </row>
     <row r="98" ht="22" customHeight="1">
       <c r="A98" s="13" t="inlineStr">
         <is>
-          <t>TASK-AI-DS-01</t>
+          <t>TASK-FW-KIN-01</t>
         </is>
       </c>
       <c r="B98" s="13" t="inlineStr">
         <is>
-          <t>Phase 2: Dataset</t>
+          <t>Phase 4A: Firmware</t>
         </is>
       </c>
       <c r="C98" s="14" t="inlineStr">
         <is>
-          <t>AI &amp; Data</t>
+          <t>Firmware</t>
         </is>
       </c>
       <c r="D98" s="14" t="inlineStr">
         <is>
-          <t>Dataset 70/15/15 Stratification Pipeline</t>
+          <t>Kinematic Actuation Delay Timer</t>
         </is>
       </c>
       <c r="E98" s="14" t="inlineStr">
         <is>
-          <t>Partition 3,000+ candling images into 70% Train, 15% Val, 15% Test across Day 10 candling captures</t>
+          <t>Calculate Delta-t = D / v = 25cm / 12.5cm/s = 2000ms delay before servo firing</t>
         </is>
       </c>
       <c r="F98" s="14" t="inlineStr">
         <is>
-          <t>IPO Matrix / Meth</t>
+          <t>Methodology 3.4</t>
         </is>
       </c>
       <c r="G98" s="13" t="inlineStr">
@@ -5860,9 +5853,9 @@
           <t>Codex</t>
         </is>
       </c>
-      <c r="H98" s="18" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="H98" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I98" s="13" t="inlineStr">
@@ -5872,14 +5865,14 @@
       </c>
       <c r="J98" s="14" t="inlineStr">
         <is>
-          <t>test_dataset_stratification.py</t>
+          <t>esp32_actuator.ino review</t>
         </is>
       </c>
     </row>
     <row r="99" ht="22" customHeight="1">
       <c r="A99" s="16" t="inlineStr">
         <is>
-          <t>TASK-AI-DS-02</t>
+          <t>TASK-AI-DS-01</t>
         </is>
       </c>
       <c r="B99" s="16" t="inlineStr">
@@ -5894,17 +5887,17 @@
       </c>
       <c r="D99" s="17" t="inlineStr">
         <is>
-          <t>Whole-Egg YOLO Bounding Box Validator</t>
+          <t>Dataset 70/15/15 Stratification Pipeline</t>
         </is>
       </c>
       <c r="E99" s="17" t="inlineStr">
         <is>
-          <t>Verify YOLO darknet format [class_id, x, y, w, h] enclosing whole egg</t>
+          <t>Partition 3,000+ candling images into 70% Train, 15% Val, 15% Test</t>
         </is>
       </c>
       <c r="F99" s="17" t="inlineStr">
         <is>
-          <t>IPO Matrix</t>
+          <t>IPO Matrix / Meth</t>
         </is>
       </c>
       <c r="G99" s="16" t="inlineStr">
@@ -5919,19 +5912,19 @@
       </c>
       <c r="I99" s="16" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J99" s="17" t="inlineStr">
         <is>
-          <t>test_annotation_bounds.py</t>
+          <t>test_dataset_stratification.py</t>
         </is>
       </c>
     </row>
     <row r="100" ht="22" customHeight="1">
       <c r="A100" s="13" t="inlineStr">
         <is>
-          <t>TASK-AI-DS-03</t>
+          <t>TASK-AI-DS-02</t>
         </is>
       </c>
       <c r="B100" s="13" t="inlineStr">
@@ -5946,17 +5939,17 @@
       </c>
       <c r="D100" s="14" t="inlineStr">
         <is>
-          <t>Candling Transillumination Augmentations</t>
+          <t>Whole-Egg YOLO Bounding Box Validator</t>
         </is>
       </c>
       <c r="E100" s="14" t="inlineStr">
         <is>
-          <t>HSV luminance jitter (V +/-20%) and +/-15 deg rotation pipeline</t>
+          <t>Verify YOLO darknet format [class_id, x, y, w, h] enclosing whole egg</t>
         </is>
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
-          <t>Chapter 3.2</t>
+          <t>IPO Matrix</t>
         </is>
       </c>
       <c r="G100" s="13" t="inlineStr">
@@ -5971,19 +5964,19 @@
       </c>
       <c r="I100" s="13" t="inlineStr">
         <is>
-          <t>P2 - Medium</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J100" s="14" t="inlineStr">
         <is>
-          <t>test_augmentation_visuals.py</t>
+          <t>test_annotation_bounds.py</t>
         </is>
       </c>
     </row>
     <row r="101" ht="22" customHeight="1">
       <c r="A101" s="16" t="inlineStr">
         <is>
-          <t>TASK-AI-DS-04</t>
+          <t>TASK-AI-DS-03</t>
         </is>
       </c>
       <c r="B101" s="16" t="inlineStr">
@@ -5998,12 +5991,12 @@
       </c>
       <c r="D101" s="17" t="inlineStr">
         <is>
-          <t>Dataset Distribution Summary Exporter</t>
+          <t>Candling Transillumination Augmentations</t>
         </is>
       </c>
       <c r="E101" s="17" t="inlineStr">
         <is>
-          <t>Generate automated Markdown and LaTeX tables of egg counts for manuscript</t>
+          <t>HSV luminance jitter (V +/-20%) and +/-15 deg rotation pipeline</t>
         </is>
       </c>
       <c r="F101" s="17" t="inlineStr">
@@ -6028,19 +6021,19 @@
       </c>
       <c r="J101" s="17" t="inlineStr">
         <is>
-          <t>export_dataset_table.py</t>
+          <t>test_augmentation_visuals.py</t>
         </is>
       </c>
     </row>
     <row r="102" ht="22" customHeight="1">
       <c r="A102" s="13" t="inlineStr">
         <is>
-          <t>TASK-AI-TRN-01</t>
+          <t>TASK-AI-DS-04</t>
         </is>
       </c>
       <c r="B102" s="13" t="inlineStr">
         <is>
-          <t>Phase 3: AI Vision</t>
+          <t>Phase 2: Dataset</t>
         </is>
       </c>
       <c r="C102" s="14" t="inlineStr">
@@ -6050,17 +6043,17 @@
       </c>
       <c r="D102" s="14" t="inlineStr">
         <is>
-          <t>Ultralytics YOLOv8 Training Script</t>
+          <t>Dataset Distribution Summary Exporter</t>
         </is>
       </c>
       <c r="E102" s="14" t="inlineStr">
         <is>
-          <t>Implement model training pipeline with CIoU + BCE + DFL loss functions</t>
+          <t>Generate automated Markdown and LaTeX tables of egg counts for manuscript</t>
         </is>
       </c>
       <c r="F102" s="14" t="inlineStr">
         <is>
-          <t>Methodology 3.3</t>
+          <t>Chapter 3.2</t>
         </is>
       </c>
       <c r="G102" s="13" t="inlineStr">
@@ -6075,19 +6068,19 @@
       </c>
       <c r="I102" s="13" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P2 - Medium</t>
         </is>
       </c>
       <c r="J102" s="14" t="inlineStr">
         <is>
-          <t>train_yolov8.py smoke test</t>
+          <t>export_dataset_table.py</t>
         </is>
       </c>
     </row>
     <row r="103" ht="22" customHeight="1">
       <c r="A103" s="16" t="inlineStr">
         <is>
-          <t>TASK-AI-OPT-01</t>
+          <t>TASK-AI-TRN-01</t>
         </is>
       </c>
       <c r="B103" s="16" t="inlineStr">
@@ -6102,17 +6095,17 @@
       </c>
       <c r="D103" s="17" t="inlineStr">
         <is>
-          <t>ONNX FP16 Slim Export &amp; Half-Precision Graph</t>
+          <t>Ultralytics YOLOv8 Training Script</t>
         </is>
       </c>
       <c r="E103" s="17" t="inlineStr">
         <is>
-          <t>Convert PyTorch weights to ONNX FP16 slim graph for edge inference</t>
+          <t>Implement model training pipeline with CIoU + BCE + DFL loss functions</t>
         </is>
       </c>
       <c r="F103" s="17" t="inlineStr">
         <is>
-          <t>AGENTS.md Tenet 3</t>
+          <t>Methodology 3.3</t>
         </is>
       </c>
       <c r="G103" s="16" t="inlineStr">
@@ -6120,26 +6113,26 @@
           <t>Codex</t>
         </is>
       </c>
-      <c r="H103" s="15" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="H103" s="18" t="inlineStr">
+        <is>
+          <t>Backlog</t>
         </is>
       </c>
       <c r="I103" s="16" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J103" s="17" t="inlineStr">
         <is>
-          <t>export_onnx.py check</t>
+          <t>train_yolov8.py smoke test</t>
         </is>
       </c>
     </row>
     <row r="104" ht="22" customHeight="1">
       <c r="A104" s="13" t="inlineStr">
         <is>
-          <t>TASK-AI-OPT-02</t>
+          <t>TASK-AI-OPT-01</t>
         </is>
       </c>
       <c r="B104" s="13" t="inlineStr">
@@ -6154,12 +6147,12 @@
       </c>
       <c r="D104" s="14" t="inlineStr">
         <is>
-          <t>Production Weights 'edge/models/weights/best.onnx'</t>
+          <t>ONNX FP16 Slim Export &amp; Half-Precision Graph</t>
         </is>
       </c>
       <c r="E104" s="14" t="inlineStr">
         <is>
-          <t>Verified production ONNX FP16 weights ready for edge execution</t>
+          <t>Convert PyTorch weights to ONNX FP16 slim graph for edge inference</t>
         </is>
       </c>
       <c r="F104" s="14" t="inlineStr">
@@ -6184,14 +6177,14 @@
       </c>
       <c r="J104" s="14" t="inlineStr">
         <is>
-          <t>test_inference_engine_and_latency_benchmark</t>
+          <t>export_onnx.py check</t>
         </is>
       </c>
     </row>
     <row r="105" ht="22" customHeight="1">
       <c r="A105" s="16" t="inlineStr">
         <is>
-          <t>TASK-AI-LAT-01</t>
+          <t>TASK-AI-OPT-02</t>
         </is>
       </c>
       <c r="B105" s="16" t="inlineStr">
@@ -6206,17 +6199,17 @@
       </c>
       <c r="D105" s="17" t="inlineStr">
         <is>
-          <t>Edge Inference Latency Benchmark (&lt;=200ms)</t>
+          <t>Production Weights 'edge/models/weights/best.onnx'</t>
         </is>
       </c>
       <c r="E105" s="17" t="inlineStr">
         <is>
-          <t>Benchmark inference latency ensuring &lt;= 200 ms SLA on edge hardware</t>
+          <t>Verified production ONNX FP16 weights ready for edge execution</t>
         </is>
       </c>
       <c r="F105" s="17" t="inlineStr">
         <is>
-          <t>Chapter 1 Objectives</t>
+          <t>AGENTS.md Tenet 3</t>
         </is>
       </c>
       <c r="G105" s="16" t="inlineStr">
@@ -6243,7 +6236,7 @@
     <row r="106" ht="22" customHeight="1">
       <c r="A106" s="13" t="inlineStr">
         <is>
-          <t>TASK-AI-EVL-01</t>
+          <t>TASK-AI-LAT-01</t>
         </is>
       </c>
       <c r="B106" s="13" t="inlineStr">
@@ -6258,17 +6251,17 @@
       </c>
       <c r="D106" s="14" t="inlineStr">
         <is>
-          <t>Breed Subgroup Metric Evaluator</t>
+          <t>Edge Inference Latency Benchmark (&lt;=200ms)</t>
         </is>
       </c>
       <c r="E106" s="14" t="inlineStr">
         <is>
-          <t>Compute Precision, Recall, F1, mAP for IP-Itim, Khaki, and Kayumanggi</t>
+          <t>Benchmark inference latency ensuring &lt;= 200 ms SLA on edge hardware</t>
         </is>
       </c>
       <c r="F106" s="14" t="inlineStr">
         <is>
-          <t>IPO Matrix</t>
+          <t>Chapter 1 Objectives</t>
         </is>
       </c>
       <c r="G106" s="13" t="inlineStr">
@@ -6276,26 +6269,26 @@
           <t>Codex</t>
         </is>
       </c>
-      <c r="H106" s="18" t="inlineStr">
-        <is>
-          <t>Backlog</t>
+      <c r="H106" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="I106" s="13" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J106" s="14" t="inlineStr">
         <is>
-          <t>test_subgroup_metrics.py</t>
+          <t>test_inference_engine_and_latency_benchmark</t>
         </is>
       </c>
     </row>
     <row r="107" ht="22" customHeight="1">
       <c r="A107" s="16" t="inlineStr">
         <is>
-          <t>TASK-AI-EVL-02</t>
+          <t>TASK-AI-EVL-01</t>
         </is>
       </c>
       <c r="B107" s="16" t="inlineStr">
@@ -6310,12 +6303,12 @@
       </c>
       <c r="D107" s="17" t="inlineStr">
         <is>
-          <t>Candling Batch Subgroup Metric Evaluator</t>
+          <t>Breed Subgroup Metric Evaluator</t>
         </is>
       </c>
       <c r="E107" s="17" t="inlineStr">
         <is>
-          <t>Compute Precision, Recall, F1, mAP across Day 10 batches and genetic groups</t>
+          <t>Compute Precision, Recall, F1, mAP for IP-Itim, Khaki, and Kayumanggi</t>
         </is>
       </c>
       <c r="F107" s="17" t="inlineStr">
@@ -6347,7 +6340,7 @@
     <row r="108" ht="22" customHeight="1">
       <c r="A108" s="13" t="inlineStr">
         <is>
-          <t>TASK-AI-EVL-03</t>
+          <t>TASK-AI-EVL-02</t>
         </is>
       </c>
       <c r="B108" s="13" t="inlineStr">
@@ -6362,17 +6355,17 @@
       </c>
       <c r="D108" s="14" t="inlineStr">
         <is>
-          <t>2-Class Confusion Matrix &amp; PR Curve Generator</t>
+          <t>Day 10 Subgroup Metric Evaluator</t>
         </is>
       </c>
       <c r="E108" s="14" t="inlineStr">
         <is>
-          <t>Generate formal 2-class confusion matrix (Fertile, Infertile) for Chapter 4</t>
+          <t>Compute Precision, Recall, F1, and mAP across Day 10 cohorts</t>
         </is>
       </c>
       <c r="F108" s="14" t="inlineStr">
         <is>
-          <t>Chapter 4 Manuscript</t>
+          <t>IPO Matrix</t>
         </is>
       </c>
       <c r="G108" s="13" t="inlineStr">
@@ -6387,49 +6380,49 @@
       </c>
       <c r="I108" s="13" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J108" s="14" t="inlineStr">
         <is>
-          <t>generate_confusion_matrix.py</t>
+          <t>test_subgroup_metrics.py</t>
         </is>
       </c>
     </row>
     <row r="109" ht="22" customHeight="1">
       <c r="A109" s="16" t="inlineStr">
         <is>
-          <t>TASK-INT-01</t>
+          <t>TASK-AI-EVL-03</t>
         </is>
       </c>
       <c r="B109" s="16" t="inlineStr">
         <is>
-          <t>Phase 5: Integration</t>
+          <t>Phase 3: AI Vision</t>
         </is>
       </c>
       <c r="C109" s="17" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>AI &amp; Data</t>
         </is>
       </c>
       <c r="D109" s="17" t="inlineStr">
         <is>
-          <t>End-to-End Sorting Pilot Simulation</t>
+          <t>2-Class Confusion Matrix &amp; PR Curve Generator</t>
         </is>
       </c>
       <c r="E109" s="17" t="inlineStr">
         <is>
-          <t>Simulate 50-egg continuous cycle: load -&gt; index -&gt; capture -&gt; predict -&gt; divert -&gt; sync</t>
+          <t>Generate Fertile/Infertile metrics for Chapter 4</t>
         </is>
       </c>
       <c r="F109" s="17" t="inlineStr">
         <is>
-          <t>System Flowchart</t>
+          <t>Chapter 4 Manuscript</t>
         </is>
       </c>
       <c r="G109" s="16" t="inlineStr">
         <is>
-          <t>Antigravity / Codex</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="H109" s="18" t="inlineStr">
@@ -6444,14 +6437,14 @@
       </c>
       <c r="J109" s="17" t="inlineStr">
         <is>
-          <t>test_end_to_end_pilot.py</t>
+          <t>generate_confusion_matrix.py</t>
         </is>
       </c>
     </row>
     <row r="110" ht="22" customHeight="1">
       <c r="A110" s="13" t="inlineStr">
         <is>
-          <t>TASK-INT-02</t>
+          <t>TASK-INT-01</t>
         </is>
       </c>
       <c r="B110" s="13" t="inlineStr">
@@ -6466,17 +6459,17 @@
       </c>
       <c r="D110" s="14" t="inlineStr">
         <is>
-          <t>Offline Network Replay Resilience Test</t>
+          <t>End-to-End Sorting Pilot Simulation</t>
         </is>
       </c>
       <c r="E110" s="14" t="inlineStr">
         <is>
-          <t>Cut network; confirm 100% sorting at edge; reconnect and verify bulk replay</t>
+          <t>Simulate 50-egg continuous cycle: load -&gt; index -&gt; capture -&gt; predict -&gt; divert -&gt; sync</t>
         </is>
       </c>
       <c r="F110" s="14" t="inlineStr">
         <is>
-          <t>AGENTS.md Offline</t>
+          <t>System Flowchart</t>
         </is>
       </c>
       <c r="G110" s="13" t="inlineStr">
@@ -6496,14 +6489,14 @@
       </c>
       <c r="J110" s="14" t="inlineStr">
         <is>
-          <t>test_offline_network_replay.py</t>
+          <t>test_end_to_end_pilot.py</t>
         </is>
       </c>
     </row>
     <row r="111" ht="22" customHeight="1">
       <c r="A111" s="16" t="inlineStr">
         <is>
-          <t>TASK-INT-03</t>
+          <t>TASK-INT-02</t>
         </is>
       </c>
       <c r="B111" s="16" t="inlineStr">
@@ -6518,17 +6511,17 @@
       </c>
       <c r="D111" s="17" t="inlineStr">
         <is>
-          <t>Cradle Position Jam Recovery Test</t>
+          <t>Offline Network Replay Resilience Test</t>
         </is>
       </c>
       <c r="E111" s="17" t="inlineStr">
         <is>
-          <t>Simulate mechanical index slip; verify conveyor pauses and resyncs</t>
+          <t>Cut network; confirm 100% sorting at edge; reconnect and verify bulk replay</t>
         </is>
       </c>
       <c r="F111" s="17" t="inlineStr">
         <is>
-          <t>System Flowchart Node 16</t>
+          <t>AGENTS.md Offline</t>
         </is>
       </c>
       <c r="G111" s="16" t="inlineStr">
@@ -6543,49 +6536,49 @@
       </c>
       <c r="I111" s="16" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J111" s="17" t="inlineStr">
         <is>
-          <t>test_cradle_resync_handler.py</t>
+          <t>test_offline_network_replay.py</t>
         </is>
       </c>
     </row>
     <row r="112" ht="22" customHeight="1">
       <c r="A112" s="13" t="inlineStr">
         <is>
-          <t>TASK-EVL-01</t>
+          <t>TASK-INT-03</t>
         </is>
       </c>
       <c r="B112" s="13" t="inlineStr">
         <is>
-          <t>Phase 6: Evaluation</t>
+          <t>Phase 5: Integration</t>
         </is>
       </c>
       <c r="C112" s="14" t="inlineStr">
         <is>
-          <t>Evaluation</t>
+          <t>Integration</t>
         </is>
       </c>
       <c r="D112" s="14" t="inlineStr">
         <is>
-          <t>Physical Sorting Accuracy Benchmark</t>
+          <t>Cradle Position Jam Recovery Test</t>
         </is>
       </c>
       <c r="E112" s="14" t="inlineStr">
         <is>
-          <t>Run &gt;= 100 physical duck egg trials to measure sorting accuracy rate</t>
+          <t>Simulate mechanical index slip; verify conveyor pauses and resyncs</t>
         </is>
       </c>
       <c r="F112" s="14" t="inlineStr">
         <is>
-          <t>Chapter 1 Objectives</t>
+          <t>System Flowchart Node 16</t>
         </is>
       </c>
       <c r="G112" s="13" t="inlineStr">
         <is>
-          <t>Antigravity</t>
+          <t>Antigravity / Codex</t>
         </is>
       </c>
       <c r="H112" s="18" t="inlineStr">
@@ -6595,19 +6588,19 @@
       </c>
       <c r="I112" s="13" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J112" s="14" t="inlineStr">
         <is>
-          <t>Physical trial tally sheet</t>
+          <t>test_cradle_resync_handler.py</t>
         </is>
       </c>
     </row>
     <row r="113" ht="22" customHeight="1">
       <c r="A113" s="16" t="inlineStr">
         <is>
-          <t>TASK-EVL-02</t>
+          <t>TASK-EVL-01</t>
         </is>
       </c>
       <c r="B113" s="16" t="inlineStr">
@@ -6622,12 +6615,12 @@
       </c>
       <c r="D113" s="17" t="inlineStr">
         <is>
-          <t>System Throughput &amp; Cycle Time Profiling</t>
+          <t>Physical Sorting Accuracy Benchmark</t>
         </is>
       </c>
       <c r="E113" s="17" t="inlineStr">
         <is>
-          <t>Measure end-to-end cycle time per egg and throughput (eggs/min)</t>
+          <t>Run &gt;= 100 physical duck egg trials to measure sorting accuracy rate</t>
         </is>
       </c>
       <c r="F113" s="17" t="inlineStr">
@@ -6647,44 +6640,44 @@
       </c>
       <c r="I113" s="16" t="inlineStr">
         <is>
-          <t>P1 - High</t>
+          <t>P0 - Critical</t>
         </is>
       </c>
       <c r="J113" s="17" t="inlineStr">
         <is>
-          <t>Kinematics benchmark report</t>
+          <t>Physical trial tally sheet</t>
         </is>
       </c>
     </row>
     <row r="114" ht="22" customHeight="1">
       <c r="A114" s="13" t="inlineStr">
         <is>
-          <t>TASK-DEF-01</t>
+          <t>TASK-EVL-02</t>
         </is>
       </c>
       <c r="B114" s="13" t="inlineStr">
         <is>
-          <t>Phase 7: Defense</t>
+          <t>Phase 6: Evaluation</t>
         </is>
       </c>
       <c r="C114" s="14" t="inlineStr">
         <is>
-          <t>Defense Prep</t>
+          <t>Evaluation</t>
         </is>
       </c>
       <c r="D114" s="14" t="inlineStr">
         <is>
-          <t>Manuscript Chapter 4 (Results &amp; Discussion)</t>
+          <t>System Throughput &amp; Cycle Time Profiling</t>
         </is>
       </c>
       <c r="E114" s="14" t="inlineStr">
         <is>
-          <t>Draft Chapter 4 using empirical metrics, confusion matrices, latency charts</t>
+          <t>Measure end-to-end cycle time per egg and throughput (eggs/min)</t>
         </is>
       </c>
       <c r="F114" s="14" t="inlineStr">
         <is>
-          <t>Chapter 4</t>
+          <t>Chapter 1 Objectives</t>
         </is>
       </c>
       <c r="G114" s="13" t="inlineStr">
@@ -6699,19 +6692,19 @@
       </c>
       <c r="I114" s="13" t="inlineStr">
         <is>
-          <t>P0 - Critical</t>
+          <t>P1 - High</t>
         </is>
       </c>
       <c r="J114" s="14" t="inlineStr">
         <is>
-          <t>Manuscript peer review</t>
+          <t>Kinematics benchmark report</t>
         </is>
       </c>
     </row>
     <row r="115" ht="22" customHeight="1">
       <c r="A115" s="16" t="inlineStr">
         <is>
-          <t>TASK-DEF-02</t>
+          <t>TASK-DEF-01</t>
         </is>
       </c>
       <c r="B115" s="16" t="inlineStr">
@@ -6726,17 +6719,17 @@
       </c>
       <c r="D115" s="17" t="inlineStr">
         <is>
-          <t>Manuscript Chapter 5 (Conclusions &amp; Recommendations)</t>
+          <t>Manuscript Chapter 4 (Results &amp; Discussion)</t>
         </is>
       </c>
       <c r="E115" s="17" t="inlineStr">
         <is>
-          <t>Summarize findings, answer research questions 1-4, formulate recommendations</t>
+          <t>Draft Chapter 4 using empirical metrics, confusion matrices, latency charts</t>
         </is>
       </c>
       <c r="F115" s="17" t="inlineStr">
         <is>
-          <t>Chapter 5</t>
+          <t>Chapter 4</t>
         </is>
       </c>
       <c r="G115" s="16" t="inlineStr">
@@ -6756,57 +6749,109 @@
       </c>
       <c r="J115" s="17" t="inlineStr">
         <is>
-          <t>Adviser review</t>
+          <t>Manuscript peer review</t>
         </is>
       </c>
     </row>
     <row r="116" ht="22" customHeight="1">
       <c r="A116" s="13" t="inlineStr">
         <is>
+          <t>TASK-DEF-02</t>
+        </is>
+      </c>
+      <c r="B116" s="13" t="inlineStr">
+        <is>
+          <t>Phase 7: Defense</t>
+        </is>
+      </c>
+      <c r="C116" s="14" t="inlineStr">
+        <is>
+          <t>Defense Prep</t>
+        </is>
+      </c>
+      <c r="D116" s="14" t="inlineStr">
+        <is>
+          <t>Manuscript Chapter 5 (Conclusions &amp; Recommendations)</t>
+        </is>
+      </c>
+      <c r="E116" s="14" t="inlineStr">
+        <is>
+          <t>Summarize findings, answer research questions 1-4, formulate recommendations</t>
+        </is>
+      </c>
+      <c r="F116" s="14" t="inlineStr">
+        <is>
+          <t>Chapter 5</t>
+        </is>
+      </c>
+      <c r="G116" s="13" t="inlineStr">
+        <is>
+          <t>Antigravity</t>
+        </is>
+      </c>
+      <c r="H116" s="18" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="I116" s="13" t="inlineStr">
+        <is>
+          <t>P0 - Critical</t>
+        </is>
+      </c>
+      <c r="J116" s="14" t="inlineStr">
+        <is>
+          <t>Adviser review</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="22" customHeight="1">
+      <c r="A117" s="16" t="inlineStr">
+        <is>
           <t>TASK-DEF-03</t>
         </is>
       </c>
-      <c r="B116" s="13" t="inlineStr">
+      <c r="B117" s="16" t="inlineStr">
         <is>
           <t>Phase 7: Defense</t>
         </is>
       </c>
-      <c r="C116" s="14" t="inlineStr">
+      <c r="C117" s="17" t="inlineStr">
         <is>
           <t>Deployment</t>
         </is>
       </c>
-      <c r="D116" s="14" t="inlineStr">
+      <c r="D117" s="17" t="inlineStr">
         <is>
           <t>1-Click Docker Production Verification</t>
         </is>
       </c>
-      <c r="E116" s="14" t="inlineStr">
+      <c r="E117" s="17" t="inlineStr">
         <is>
           <t>Verify docker-compose up for PostgreSQL 16, FastAPI backend, React dashboard</t>
         </is>
       </c>
-      <c r="F116" s="14" t="inlineStr">
+      <c r="F117" s="17" t="inlineStr">
         <is>
           <t>docker-compose.yml</t>
         </is>
       </c>
-      <c r="G116" s="13" t="inlineStr">
+      <c r="G117" s="16" t="inlineStr">
         <is>
           <t>Antigravity / Codex</t>
         </is>
       </c>
-      <c r="H116" s="15" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="I116" s="13" t="inlineStr">
+      <c r="H117" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I117" s="16" t="inlineStr">
         <is>
           <t>P0 - Critical</t>
         </is>
       </c>
-      <c r="J116" s="14" t="inlineStr">
+      <c r="J117" s="17" t="inlineStr">
         <is>
           <t>docker-compose config test</t>
         </is>

</xml_diff>

<commit_message>
feat(firmware): integrate egg and servo prototype controls
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -152,7 +152,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -199,6 +199,15 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -862,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J117"/>
+  <dimension ref="A3:J118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6857,6 +6866,58 @@
         </is>
       </c>
     </row>
+    <row r="118" ht="60" customHeight="1">
+      <c r="A118" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-FW-APP-01</t>
+        </is>
+      </c>
+      <c r="B118" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4A: Firmware</t>
+        </is>
+      </c>
+      <c r="C118" s="20" t="inlineStr">
+        <is>
+          <t>Firmware</t>
+        </is>
+      </c>
+      <c r="D118" s="20" t="inlineStr">
+        <is>
+          <t>Unified egg and servo prototype app</t>
+        </is>
+      </c>
+      <c r="E118" s="20" t="inlineStr">
+        <is>
+          <t>CustomTkinter app with independent serial workers, calibration, servo presets, shared controls and explicit simulation</t>
+        </is>
+      </c>
+      <c r="F118" s="20" t="inlineStr">
+        <is>
+          <t>Firmware prototype</t>
+        </is>
+      </c>
+      <c r="G118" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H118" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I118" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J118" s="20" t="inlineStr">
+        <is>
+          <t>edge/tests/test_firmware_prototype.py + GUI simulation smoke test</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(firmware): optimize operator workspace and add egg detection
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J118"/>
+  <dimension ref="A3:J119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6918,6 +6918,58 @@
         </is>
       </c>
     </row>
+    <row r="119" ht="60" customHeight="1">
+      <c r="A119" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-FW-DET-01</t>
+        </is>
+      </c>
+      <c r="B119" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4A: Firmware</t>
+        </is>
+      </c>
+      <c r="C119" s="20" t="inlineStr">
+        <is>
+          <t>Firmware</t>
+        </is>
+      </c>
+      <c r="D119" s="20" t="inlineStr">
+        <is>
+          <t>Camera egg detection and optimized operator workspace</t>
+        </is>
+      </c>
+      <c r="E119" s="20" t="inlineStr">
+        <is>
+          <t>Real ONNX classification, stable egg presence, WAL scan recording, manual review, optical events, and bounded background work</t>
+        </is>
+      </c>
+      <c r="F119" s="20" t="inlineStr">
+        <is>
+          <t>Edge prototype</t>
+        </is>
+      </c>
+      <c r="G119" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H119" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I119" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J119" s="20" t="inlineStr">
+        <is>
+          <t>edge/tests/test_prototype_vision.py and real camera UI smoke test</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(firmware): add automatic stepper camera and servo cycle
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J119"/>
+  <dimension ref="A3:J120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6970,6 +6970,58 @@
         </is>
       </c>
     </row>
+    <row r="120" ht="60" customHeight="1">
+      <c r="A120" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-FW-CYCLE-01</t>
+        </is>
+      </c>
+      <c r="B120" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4A: Firmware</t>
+        </is>
+      </c>
+      <c r="C120" s="20" t="inlineStr">
+        <is>
+          <t>Firmware</t>
+        </is>
+      </c>
+      <c r="D120" s="20" t="inlineStr">
+        <is>
+          <t>Automatic stepper, camera and servo integration cycle</t>
+        </is>
+      </c>
+      <c r="E120" s="20" t="inlineStr">
+        <is>
+          <t>Configurable travel, stationary captures, persisted detection, feedback-driven moves, gate hold, repeat cycles, and manual-review recovery</t>
+        </is>
+      </c>
+      <c r="F120" s="20" t="inlineStr">
+        <is>
+          <t>Edge prototype</t>
+        </is>
+      </c>
+      <c r="G120" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H120" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I120" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J120" s="20" t="inlineStr">
+        <is>
+          <t>edge/tests/test_prototype_cycle.py, inspection rearm tests and UI smoke check</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(edge): integrate dual-board sorting and camera defaults
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J120"/>
+  <dimension ref="A3:J121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7022,6 +7022,58 @@
         </is>
       </c>
     </row>
+    <row r="121" ht="70" customHeight="1">
+      <c r="A121" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-CONTROL-01</t>
+        </is>
+      </c>
+      <c r="B121" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C121" s="20" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D121" s="20" t="inlineStr">
+        <is>
+          <t>Dual-board station control and camera defaults</t>
+        </is>
+      </c>
+      <c r="E121" s="20" t="inlineStr">
+        <is>
+          <t>IR-stopped holder tracking; WAL evidence; saved camera/AI defaults. Firmware identification, upload and rig bench validation remain required.</t>
+        </is>
+      </c>
+      <c r="F121" s="20" t="inlineStr">
+        <is>
+          <t>docs/OVALENS_EDGE_STATION_CONTROL.md</t>
+        </is>
+      </c>
+      <c r="G121" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H121" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I121" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J121" s="20" t="inlineStr">
+        <is>
+          <t>edge/tests/test_station_control.py; native firmware tests; hidden-window UI tests</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(edge): improve operator typography and status performance
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J121"/>
+  <dimension ref="A3:J122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7074,6 +7074,58 @@
         </is>
       </c>
     </row>
+    <row r="122" ht="70" customHeight="1">
+      <c r="A122" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-UI-POLISH-01</t>
+        </is>
+      </c>
+      <c r="B122" s="19" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="C122" s="20" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D122" s="20" t="inlineStr">
+        <is>
+          <t>Operator typography and visibility</t>
+        </is>
+      </c>
+      <c r="E122" s="20" t="inlineStr">
+        <is>
+          <t>Native Segoe UI; readable status, controls and settings; minimum 1024x720 layout; skip unchanged Tk control and HUD updates. Simulated GUI and before/after status benchmark.</t>
+        </is>
+      </c>
+      <c r="F122" s="20" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-CONTROL-01</t>
+        </is>
+      </c>
+      <c r="G122" s="19" t="inlineStr">
+        <is>
+          <t>Operator</t>
+        </is>
+      </c>
+      <c r="H122" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I122" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J122" s="20" t="inlineStr">
+        <is>
+          <t>test_ui_refresh.py; test_startup_config.py; repository verification gate</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor(edge): focus operator design on camera and sorting
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J122"/>
+  <dimension ref="A3:J123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7126,6 +7126,58 @@
         </is>
       </c>
     </row>
+    <row r="123" ht="70" customHeight="1">
+      <c r="A123" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-DESIGN-02</t>
+        </is>
+      </c>
+      <c r="B123" s="19" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="C123" s="20" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D123" s="20" t="inlineStr">
+        <is>
+          <t>Focused operator design with impeccable</t>
+        </is>
+      </c>
+      <c r="E123" s="20" t="inlineStr">
+        <is>
+          <t>Single record panel; count rows; restrained semantic colour; camera empty state; primary versus secondary actions. Preserve cached refreshes and minimum-size review controls.</t>
+        </is>
+      </c>
+      <c r="F123" s="20" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-CONTROL-01</t>
+        </is>
+      </c>
+      <c r="G123" s="19" t="inlineStr">
+        <is>
+          <t>Operator</t>
+        </is>
+      </c>
+      <c r="H123" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I123" s="19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J123" s="20" t="inlineStr">
+        <is>
+          <t>test_ui_refresh.py; test_startup_config.py; repository verification gate</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(edge): integrate three-board candling rig
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J123"/>
+  <dimension ref="A3:J124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7178,6 +7178,58 @@
         </is>
       </c>
     </row>
+    <row r="124" ht="80" customHeight="1">
+      <c r="A124" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-3BOARD-01</t>
+        </is>
+      </c>
+      <c r="B124" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C124" s="20" t="inlineStr">
+        <is>
+          <t>Edge CV</t>
+        </is>
+      </c>
+      <c r="D124" s="20" t="inlineStr">
+        <is>
+          <t>Three-board candling integration</t>
+        </is>
+      </c>
+      <c r="E124" s="20" t="inlineStr">
+        <is>
+          <t>Versioned discovery; hardware pause; fresh capture; WAL evidence; position-tracked gates; manual review and recovery. Firmware upload, intended model and physical acceptance remain separately required.</t>
+        </is>
+      </c>
+      <c r="F124" s="20" t="inlineStr">
+        <is>
+          <t>docs/EDGE_THREE_BOARD_IMPLEMENTATION.md</t>
+        </is>
+      </c>
+      <c r="G124" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H124" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I124" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J124" s="20" t="inlineStr">
+        <is>
+          <t>50-egg worker simulation; native firmware tests; ESP32 builds; repository verification gate</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(edge): simplify default station setup
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J124"/>
+  <dimension ref="A3:J125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7230,6 +7230,58 @@
         </is>
       </c>
     </row>
+    <row r="125" ht="80" customHeight="1">
+      <c r="A125" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-SETUP-01</t>
+        </is>
+      </c>
+      <c r="B125" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C125" s="20" t="inlineStr">
+        <is>
+          <t>Edge CV</t>
+        </is>
+      </c>
+      <c r="D125" s="20" t="inlineStr">
+        <is>
+          <t>Simple default station setup</t>
+        </is>
+      </c>
+      <c r="E125" s="20" t="inlineStr">
+        <is>
+          <t>Remember COM5 stepper, COM7 servo + IR and COM9 light; role detection; main-screen empty-conveyor preparation; cancellable background setup.</t>
+        </is>
+      </c>
+      <c r="F125" s="20" t="inlineStr">
+        <is>
+          <t>docs/EDGE_THREE_BOARD_IMPLEMENTATION.md</t>
+        </is>
+      </c>
+      <c r="G125" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H125" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I125" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J125" s="20" t="inlineStr">
+        <is>
+          <t>Transport, persistence, cancellation and native GUI tests; repository quality gate; no hardware access</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(edge): select project Python before loading packages
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J125"/>
+  <dimension ref="A3:J126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7282,6 +7282,58 @@
         </is>
       </c>
     </row>
+    <row r="126" ht="80" customHeight="1">
+      <c r="A126" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-RUNTIME-01</t>
+        </is>
+      </c>
+      <c r="B126" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C126" s="20" t="inlineStr">
+        <is>
+          <t>Edge CV</t>
+        </is>
+      </c>
+      <c r="D126" s="20" t="inlineStr">
+        <is>
+          <t>Select project Python at launch</t>
+        </is>
+      </c>
+      <c r="E126" s="20" t="inlineStr">
+        <is>
+          <t>Prefer .venv before dependency imports; double-click Windows launcher; hardware-free runtime check; avoid serial package collision.</t>
+        </is>
+      </c>
+      <c r="F126" s="20" t="inlineStr">
+        <is>
+          <t>edge/README.md</t>
+        </is>
+      </c>
+      <c r="G126" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H126" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I126" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J126" s="20" t="inlineStr">
+        <is>
+          <t>Interpreter bootstrap unit tests; real global-to-venv import check; repository quality gate</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(firmware): install and verify three-board v3 builds
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J126"/>
+  <dimension ref="A3:J127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7334,6 +7334,58 @@
         </is>
       </c>
     </row>
+    <row r="127" ht="80" customHeight="1">
+      <c r="A127" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-FW-INSTALL-01</t>
+        </is>
+      </c>
+      <c r="B127" s="19" t="inlineStr">
+        <is>
+          <t>Phase 5: Firmware</t>
+        </is>
+      </c>
+      <c r="C127" s="20" t="inlineStr">
+        <is>
+          <t>Firmware</t>
+        </is>
+      </c>
+      <c r="D127" s="20" t="inlineStr">
+        <is>
+          <t>Install three-board v3 firmware</t>
+        </is>
+      </c>
+      <c r="E127" s="20" t="inlineStr">
+        <is>
+          <t>Explicit user approval with empty conveyor; identify old firmware; rebuild and upload COM5/7/9; verify flash hashes, v3 roles and paused/lamp-off telemetry. Physical sorting remains untested.</t>
+        </is>
+      </c>
+      <c r="F127" s="20" t="inlineStr">
+        <is>
+          <t>docs/EDGE_THREE_BOARD_IMPLEMENTATION.md</t>
+        </is>
+      </c>
+      <c r="G127" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H127" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I127" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J127" s="20" t="inlineStr">
+        <is>
+          <t>Three ESP32 builds; three verified uploads; actual application discovery and boot telemetry</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
perf(edge): classify only confirmed stopped eggs
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J127"/>
+  <dimension ref="A3:J128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7386,6 +7386,58 @@
         </is>
       </c>
     </row>
+    <row r="128" ht="80" customHeight="1">
+      <c r="A128" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-STOPSCAN-01</t>
+        </is>
+      </c>
+      <c r="B128" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C128" s="20" t="inlineStr">
+        <is>
+          <t>Edge CV</t>
+        </is>
+      </c>
+      <c r="D128" s="20" t="inlineStr">
+        <is>
+          <t>Infer only on stopped eggs</t>
+        </is>
+      </c>
+      <c r="E128" s="20" t="inlineStr">
+        <is>
+          <t>Live preview without continuous inference; confirmed stop; three samples across 300ms; paired captured image and detections; clear before motion.</t>
+        </is>
+      </c>
+      <c r="F128" s="20" t="inlineStr">
+        <is>
+          <t>edge/README.md</t>
+        </is>
+      </c>
+      <c r="G128" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H128" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I128" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J128" s="20" t="inlineStr">
+        <is>
+          <t>Simulated stopped capture, cancellation, exact frame evidence and 50-egg worker/WAL tests; repository quality gate</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(edge): position sorting gate before conveyor release
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J128"/>
+  <dimension ref="A3:J129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7438,6 +7438,58 @@
         </is>
       </c>
     </row>
+    <row r="129" ht="80" customHeight="1">
+      <c r="A129" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-GATEFIRST-01</t>
+        </is>
+      </c>
+      <c r="B129" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C129" s="20" t="inlineStr">
+        <is>
+          <t>Edge CV</t>
+        </is>
+      </c>
+      <c r="D129" s="20" t="inlineStr">
+        <is>
+          <t>Position sorting gate before conveyor release</t>
+        </is>
+      </c>
+      <c r="E129" s="20" t="inlineStr">
+        <is>
+          <t>Durable classification, confirmed servo completion, then conveyor release; retain gate until calibrated exit; protect earlier eggs on premature arrivals.</t>
+        </is>
+      </c>
+      <c r="F129" s="20" t="inlineStr">
+        <is>
+          <t>edge/README.md</t>
+        </is>
+      </c>
+      <c r="G129" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H129" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I129" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J129" s="20" t="inlineStr">
+        <is>
+          <t>Command ordering, blocked servo completion, servo failures, premature arrivals, exact exit boundary, and full repository gate</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(edge): simplify daily operator workflow
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J129"/>
+  <dimension ref="A3:J130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7490,6 +7490,58 @@
         </is>
       </c>
     </row>
+    <row r="130" ht="80" customHeight="1">
+      <c r="A130" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-EASYFLOW-01</t>
+        </is>
+      </c>
+      <c r="B130" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C130" s="20" t="inlineStr">
+        <is>
+          <t>Edge CV</t>
+        </is>
+      </c>
+      <c r="D130" s="20" t="inlineStr">
+        <is>
+          <t>Simplify daily edge operation</t>
+        </is>
+      </c>
+      <c r="E130" s="20" t="inlineStr">
+        <is>
+          <t>One inspected Start sorting action; remembered settings; live preview; feeding cues; Tools diagnostics; inline automatic completion; shorter default display hold.</t>
+        </is>
+      </c>
+      <c r="F130" s="20" t="inlineStr">
+        <is>
+          <t>edge/README.md</t>
+        </is>
+      </c>
+      <c r="G130" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H130" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I130" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J130" s="20" t="inlineStr">
+        <is>
+          <t>Combined startup/cancellation, preserved calibration, completion/retry, state cues and native GUI checks; full repository gate</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(edge): allow longer settling before egg capture
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J130"/>
+  <dimension ref="A3:J131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7542,6 +7542,58 @@
         </is>
       </c>
     </row>
+    <row r="131" ht="80" customHeight="1">
+      <c r="A131" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-CAPTURE-SETTLE-01</t>
+        </is>
+      </c>
+      <c r="B131" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C131" s="20" t="inlineStr">
+        <is>
+          <t>Edge CV</t>
+        </is>
+      </c>
+      <c r="D131" s="20" t="inlineStr">
+        <is>
+          <t>Allow egg and camera to settle before capture</t>
+        </is>
+      </c>
+      <c r="E131" s="20" t="inlineStr">
+        <is>
+          <t>1500ms pre-capture default; preserve custom settings, confidence, buffer flush and gate ordering; verify capture order and STOP.</t>
+        </is>
+      </c>
+      <c r="F131" s="20" t="inlineStr">
+        <is>
+          <t>docs/EDGE_THREE_BOARD_IMPLEMENTATION.md</t>
+        </is>
+      </c>
+      <c r="G131" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H131" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I131" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J131" s="20" t="inlineStr">
+        <is>
+          <t>Software capture-order and cancellation regressions; physical sharpness pending operator trial</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(edge): use verified best_v3 model export
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J131"/>
+  <dimension ref="A3:J132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7594,6 +7594,58 @@
         </is>
       </c>
     </row>
+    <row r="132" ht="80" customHeight="1">
+      <c r="A132" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-MODEL-V3-01</t>
+        </is>
+      </c>
+      <c r="B132" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C132" s="20" t="inlineStr">
+        <is>
+          <t>Edge CV</t>
+        </is>
+      </c>
+      <c r="D132" s="20" t="inlineStr">
+        <is>
+          <t>Integrate supplied best_v3 detector</t>
+        </is>
+      </c>
+      <c r="E132" s="20" t="inlineStr">
+        <is>
+          <t>Verified ONNX export of supplied checkpoint; prefer v3, retain explicit overrides and prior model; offline validation and benchmark.</t>
+        </is>
+      </c>
+      <c r="F132" s="20" t="inlineStr">
+        <is>
+          <t>docs/EDGE_THREE_BOARD_IMPLEMENTATION.md</t>
+        </is>
+      </c>
+      <c r="G132" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H132" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I132" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J132" s="20" t="inlineStr">
+        <is>
+          <t>Contract, path precedence, empty-image and saved-capture smoke checks; full gate; accuracy requires labelled validation</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(edge): tune camera beside live preview
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J132"/>
+  <dimension ref="A3:J133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7646,6 +7646,58 @@
         </is>
       </c>
     </row>
+    <row r="133" ht="80" customHeight="1">
+      <c r="A133" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-CAMERA-PREVIEW-01</t>
+        </is>
+      </c>
+      <c r="B133" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C133" s="20" t="inlineStr">
+        <is>
+          <t>Edge CV</t>
+        </is>
+      </c>
+      <c r="D133" s="20" t="inlineStr">
+        <is>
+          <t>Tune camera beside live preview</t>
+        </is>
+      </c>
+      <c r="E133" s="20" t="inlineStr">
+        <is>
+          <t>Idle preview camera controls with automatic modes, image properties, readback and save; no serial commands.</t>
+        </is>
+      </c>
+      <c r="F133" s="20" t="inlineStr">
+        <is>
+          <t>edge/README.md</t>
+        </is>
+      </c>
+      <c r="G133" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H133" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I133" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J133" s="20" t="inlineStr">
+        <is>
+          <t>Fake camera ownership, apply/save/failure, operation guards and native minimum-size preview checks</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(edge): add camera sliders and cradle alignment
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J133"/>
+  <dimension ref="A3:J134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7698,6 +7698,38 @@
         </is>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-CAMERA-ALIGN-01</t>
+        </is>
+      </c>
+      <c r="B134" s="19" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="C134" s="20" t="inlineStr">
+        <is>
+          <t>Camera sliders and cradle alignment</t>
+        </is>
+      </c>
+      <c r="D134" s="20" t="inlineStr">
+        <is>
+          <t>Editable saved camera slider spans and bounded idle stepper jog controls</t>
+        </is>
+      </c>
+      <c r="E134" s="20" t="n"/>
+      <c r="F134" s="20" t="n"/>
+      <c r="G134" s="19" t="n"/>
+      <c r="H134" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I134" s="19" t="n"/>
+      <c r="J134" s="20" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(edge): apply camera preview tweaks live
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J134"/>
+  <dimension ref="A3:J135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7730,6 +7730,38 @@
       <c r="I134" s="19" t="n"/>
       <c r="J134" s="20" t="n"/>
     </row>
+    <row r="135">
+      <c r="A135" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-CAMERA-LIVE-01</t>
+        </is>
+      </c>
+      <c r="B135" s="19" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="C135" s="20" t="inlineStr">
+        <is>
+          <t>Live camera tuning</t>
+        </is>
+      </c>
+      <c r="D135" s="20" t="inlineStr">
+        <is>
+          <t>Coalesced preview adjustments, frame continuity and explicit persistence</t>
+        </is>
+      </c>
+      <c r="E135" s="20" t="n"/>
+      <c r="F135" s="20" t="n"/>
+      <c r="G135" s="19" t="n"/>
+      <c r="H135" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I135" s="19" t="n"/>
+      <c r="J135" s="20" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(edge): sync saved scan images to backend
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J135"/>
+  <dimension ref="A3:J136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7762,6 +7762,58 @@
       <c r="I135" s="19" t="n"/>
       <c r="J135" s="20" t="n"/>
     </row>
+    <row r="136" ht="80" customHeight="1">
+      <c r="A136" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-IMAGE-SYNC-01</t>
+        </is>
+      </c>
+      <c r="B136" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C136" s="20" t="inlineStr">
+        <is>
+          <t>Edge / Backend</t>
+        </is>
+      </c>
+      <c r="D136" s="20" t="inlineStr">
+        <is>
+          <t>Save and sync scan photos</t>
+        </is>
+      </c>
+      <c r="E136" s="20" t="inlineStr">
+        <is>
+          <t>Paired local JPEG evidence, durable image outbox, validated atomic backend uploads and dashboard media routing</t>
+        </is>
+      </c>
+      <c r="F136" s="20" t="inlineStr">
+        <is>
+          <t>edge/README.md</t>
+        </is>
+      </c>
+      <c r="G136" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H136" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I136" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J136" s="20" t="inlineStr">
+        <is>
+          <t>Image replay, failure recovery, API storage and full repository gate</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(edge): add manual candling light switch
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J136"/>
+  <dimension ref="A3:J137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7814,6 +7814,58 @@
         </is>
       </c>
     </row>
+    <row r="137" ht="80" customHeight="1">
+      <c r="A137" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-MANUAL-LIGHT-01</t>
+        </is>
+      </c>
+      <c r="B137" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C137" s="20" t="inlineStr">
+        <is>
+          <t>Edge CV</t>
+        </is>
+      </c>
+      <c r="D137" s="20" t="inlineStr">
+        <is>
+          <t>Manual candling light switch</t>
+        </is>
+      </c>
+      <c r="E137" s="20" t="inlineStr">
+        <is>
+          <t>Confirmed on/off, lamp-only COM9 connection, watchdog renewal, operation locks and STOP cancellation</t>
+        </is>
+      </c>
+      <c r="F137" s="20" t="inlineStr">
+        <is>
+          <t>edge/README.md</t>
+        </is>
+      </c>
+      <c r="G137" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H137" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I137" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J137" s="20" t="inlineStr">
+        <is>
+          <t>Verified: 27 backend tests; 406 Edge passed + 1 shared-Tk skip passed in a fresh process; dashboard build. Fake lamp connection, renewal, cancellation, retry, handoff and native 1024/1280 layout checks. No physical hardware operated.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(edge): pause and resume active sorting sessions
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J137"/>
+  <dimension ref="A3:J138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7866,6 +7866,58 @@
         </is>
       </c>
     </row>
+    <row r="138" ht="80" customHeight="1">
+      <c r="A138" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-PAUSE-01</t>
+        </is>
+      </c>
+      <c r="B138" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C138" s="20" t="inlineStr">
+        <is>
+          <t>Edge CV</t>
+        </is>
+      </c>
+      <c r="D138" s="20" t="inlineStr">
+        <is>
+          <t>Pause and resume sorting</t>
+        </is>
+      </c>
+      <c r="E138" s="20" t="inlineStr">
+        <is>
+          <t>Same-session stopped-boundary hold, durable scans and photos, gate/position validation and jam deadline suspension</t>
+        </is>
+      </c>
+      <c r="F138" s="20" t="inlineStr">
+        <is>
+          <t>edge/README.md</t>
+        </is>
+      </c>
+      <c r="G138" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H138" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I138" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J138" s="20" t="inlineStr">
+        <is>
+          <t>Verified: 27 backend tests, 422 Edge tests and dashboard build. Repeated pause/resume, saved photos/counts, unchanged session and sequence, hold validation, STOP, jam timeout suspension, and native 1024/1280 controls. No physical hardware operated.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(edge): allow automatic sorting at 70 percent confidence
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J138"/>
+  <dimension ref="A3:J139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7918,6 +7918,58 @@
         </is>
       </c>
     </row>
+    <row r="139" ht="80" customHeight="1">
+      <c r="A139" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-CONFIDENCE-70-01</t>
+        </is>
+      </c>
+      <c r="B139" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C139" s="20" t="inlineStr">
+        <is>
+          <t>Edge / Backend</t>
+        </is>
+      </c>
+      <c r="D139" s="20" t="inlineStr">
+        <is>
+          <t>Automatic sorting at 70% confidence</t>
+        </is>
+      </c>
+      <c r="E139" s="20" t="inlineStr">
+        <is>
+          <t>Configure this station and new defaults at 0.70; permit durable stable decisions and align backend review counts/filter; retain stricter saved thresholds and review fallback</t>
+        </is>
+      </c>
+      <c r="F139" s="20" t="inlineStr">
+        <is>
+          <t>edge/README.md</t>
+        </is>
+      </c>
+      <c r="G139" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H139" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I139" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J139" s="20" t="inlineStr">
+        <is>
+          <t>Verified: 28 backend tests, 432 Edge tests and dashboard build. Exact 70% accept/reject boundaries, review below configured thresholds, durable writes before routing, saved configuration, sync idempotency and review metrics/filtering. Software verification only.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(edge): replay completed sessions and unblock sync
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J139"/>
+  <dimension ref="A3:J140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7970,6 +7970,58 @@
         </is>
       </c>
     </row>
+    <row r="140">
+      <c r="A140" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-SESSION-SYNC-01</t>
+        </is>
+      </c>
+      <c r="B140" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C140" s="20" t="inlineStr">
+        <is>
+          <t>Edge / Dashboard</t>
+        </is>
+      </c>
+      <c r="D140" s="20" t="inlineStr">
+        <is>
+          <t>Durable session sync and dashboard completion</t>
+        </is>
+      </c>
+      <c r="E140" s="20" t="inlineStr">
+        <is>
+          <t>Retry completed session timestamps after all scan acknowledgements, survive restarts, avoid blocked-batch starvation, correct office batch selection and refresh candling history</t>
+        </is>
+      </c>
+      <c r="F140" s="20" t="inlineStr">
+        <is>
+          <t>edge/README.md</t>
+        </is>
+      </c>
+      <c r="G140" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H140" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I140" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J140" s="20" t="inlineStr">
+        <is>
+          <t>Verified: 34 backend tests, 442 Edge tests, 34 dashboard tests and production build. Lost acknowledgements, restart migration, missing-batch fairness, original session identity/time, saved office selection and preserved hatch stage. No physical hardware operated.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(edge): allow stable off-centre automatic sorting
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J140"/>
+  <dimension ref="A3:J141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8022,6 +8022,58 @@
         </is>
       </c>
     </row>
+    <row r="141">
+      <c r="A141" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-OFFCENTER-01</t>
+        </is>
+      </c>
+      <c r="B141" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C141" s="20" t="inlineStr">
+        <is>
+          <t>Edge CV</t>
+        </is>
+      </c>
+      <c r="D141" s="20" t="inlineStr">
+        <is>
+          <t>Automatic off-centre egg sorting</t>
+        </is>
+      </c>
+      <c r="E141" s="20" t="inlineStr">
+        <is>
+          <t>Remove the fixed centre-zone veto; require three stopped agreeing frames at the saved threshold, valid geometry, durable scan/photo and confirmed gate before release</t>
+        </is>
+      </c>
+      <c r="F141" s="20" t="inlineStr">
+        <is>
+          <t>edge/README.md</t>
+        </is>
+      </c>
+      <c r="G141" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H141" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I141" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J141" s="20" t="inlineStr">
+        <is>
+          <t>Verified: 34 backend tests, 461 Edge tests and dashboard production build. Recorded off-centre box sorts at 0.70, 0.81 and 0.8188 with three stopped captures, durable photos/scans and confirmed gate before release. Invalid geometry, disagreement, multiple eggs and low confidence still review. Simulated camera test holds use a finite 10-second backstop for slow Tk redraws. No physical hardware operated.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(edge): create and sync complete batches offline
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J141"/>
+  <dimension ref="A3:J142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8074,6 +8074,58 @@
         </is>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-BATCH-CREATE-01</t>
+        </is>
+      </c>
+      <c r="B142" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C142" s="20" t="inlineStr">
+        <is>
+          <t>Edge / Backend</t>
+        </is>
+      </c>
+      <c r="D142" s="20" t="inlineStr">
+        <is>
+          <t>Worker-led offline batch creation</t>
+        </is>
+      </c>
+      <c r="E142" s="20" t="inlineStr">
+        <is>
+          <t>Persist full batches and stable IDs, cached selection, remembered defaults, legacy metadata repair, idempotent registration before scans, worker create permissions and native setup verification</t>
+        </is>
+      </c>
+      <c r="F142" s="20" t="inlineStr">
+        <is>
+          <t>edge/README.md</t>
+        </is>
+      </c>
+      <c r="G142" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H142" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I142" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J142" s="20" t="inlineStr">
+        <is>
+          <t>Verified: 48 backend tests on isolated PostgreSQL, 486 Edge tests and dashboard production build. Offline creation, stable IDs, separate inventory/run targets, cached selection, legacy metadata repair, lost/conflicting/concurrent registrations, worker permissions, native 1024/1280 layouts and cross-process SQLite integrity. Farm database read-only integrity check passed. No hardware operated.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(edge): prepare and verify station before sorting
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J142"/>
+  <dimension ref="A3:J143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8126,6 +8126,58 @@
         </is>
       </c>
     </row>
+    <row r="143">
+      <c r="A143" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-READINESS-01</t>
+        </is>
+      </c>
+      <c r="B143" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C143" s="20" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D143" s="20" t="inlineStr">
+        <is>
+          <t>Station readiness before sorting</t>
+        </is>
+      </c>
+      <c r="E143" s="20" t="inlineStr">
+        <is>
+          <t>Separate passive startup checks, inspected preparation and final Start; invalidate stale readiness, preserve offline work and verify native controls without hardware</t>
+        </is>
+      </c>
+      <c r="F143" s="20" t="inlineStr">
+        <is>
+          <t>edge/README.md</t>
+        </is>
+      </c>
+      <c r="G143" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H143" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I143" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J143" s="20" t="inlineStr">
+        <is>
+          <t>Backend 48 tests and Edge regression gate passed; dashboard build passed. Native preparation, fault, offline and recovery controls verified at 1024x720 and 1280x860 with fake camera/serial. Physical hardware untouched; real actuator feedback remains a separate rig acceptance check.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(edge): add standalone COM5 stepper diagnostic
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J143"/>
+  <dimension ref="A3:J144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8178,6 +8178,58 @@
         </is>
       </c>
     </row>
+    <row r="144">
+      <c r="A144" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-STEPPER-TEST-01</t>
+        </is>
+      </c>
+      <c r="B144" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C144" s="20" t="inlineStr">
+        <is>
+          <t>Edge / Firmware</t>
+        </is>
+      </c>
+      <c r="D144" s="20" t="inlineStr">
+        <is>
+          <t>Standalone COM5 stepper diagnostic</t>
+        </is>
+      </c>
+      <c r="E144" s="20" t="inlineStr">
+        <is>
+          <t>Finite relative jog; v3 identity, pause, speed and position verification; no other ports, homing, photos or batch writes; stop on error/Ctrl+C</t>
+        </is>
+      </c>
+      <c r="F144" s="20" t="inlineStr">
+        <is>
+          <t>firmware/three_board/README.md</t>
+        </is>
+      </c>
+      <c r="G144" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H144" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I144" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J144" s="20" t="inlineStr">
+        <is>
+          <t>17 simulated stepper tests passed, including pause interlock, role, speed, position and Ctrl+C checks; backend/Edge/dashboard gate passed. COM5-only per operator request. Physical hardware was not accessed; actual motion requires pause LOW and observation.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(edge): add standalone COM7 servo diagnostic
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J144"/>
+  <dimension ref="A3:J145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8230,6 +8230,58 @@
         </is>
       </c>
     </row>
+    <row r="145">
+      <c r="A145" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-SERVO-TEST-01</t>
+        </is>
+      </c>
+      <c r="B145" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C145" s="20" t="inlineStr">
+        <is>
+          <t>Edge / Firmware</t>
+        </is>
+      </c>
+      <c r="D145" s="20" t="inlineStr">
+        <is>
+          <t>Standalone COM7 servo diagnostic</t>
+        </is>
+      </c>
+      <c r="E145" s="20" t="inlineStr">
+        <is>
+          <t>Bounded angle sequence; confirmation before boot reset, held pause, clear IR, v3 identity and angle completion; stop/close on errors and Ctrl+C</t>
+        </is>
+      </c>
+      <c r="F145" s="20" t="inlineStr">
+        <is>
+          <t>firmware/three_board/README.md</t>
+        </is>
+      </c>
+      <c r="G145" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H145" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I145" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J145" s="20" t="inlineStr">
+        <is>
+          <t>22 simulated servo checks passed: COM7-only, bounded angles, clear-path confirmation before boot reset, boot settling, held pause, blocked IR during observation, role/fault/angle validation and Ctrl+C cleanup. Backend/Edge/dashboard gate passed. Physical hardware untouched; actual movement remains an observed rig check.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(edge): remove IR requirements from servo test
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J145"/>
+  <dimension ref="A3:J146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8282,6 +8282,58 @@
         </is>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-SERVO-SIMPLE-01</t>
+        </is>
+      </c>
+      <c r="B146" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C146" s="20" t="inlineStr">
+        <is>
+          <t>Edge / Firmware</t>
+        </is>
+      </c>
+      <c r="D146" s="20" t="inlineStr">
+        <is>
+          <t>Simple servo test without IR</t>
+        </is>
+      </c>
+      <c r="E146" s="20" t="inlineStr">
+        <is>
+          <t>Visible 90/120/90 servo diagnostic independent of IR presence/readings and egg-cycle state; retain controller identity, bounded angles, held pause and cleanup</t>
+        </is>
+      </c>
+      <c r="F146" s="20" t="inlineStr">
+        <is>
+          <t>firmware/three_board/README.md</t>
+        </is>
+      </c>
+      <c r="G146" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H146" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I146" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J146" s="20" t="inlineStr">
+        <is>
+          <t>23 simulated servo checks passed, including blocked/missing/changing IR and HOLDING/CLEARING states. Full Edge run: 553 passed, two Tk skips, one existing pause-button UI failure; failed test passed on targeted gate rerun. Backend 48 and dashboard build passed. COM7-only 90/120/90, pause held; physical hardware untouched.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(edge): synchronize servo diagnostic serial startup
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J146"/>
+  <dimension ref="A3:J147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8334,6 +8334,58 @@
         </is>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-SERVO-STARTUP-01</t>
+        </is>
+      </c>
+      <c r="B147" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C147" s="20" t="inlineStr">
+        <is>
+          <t>Edge / Firmware</t>
+        </is>
+      </c>
+      <c r="D147" s="20" t="inlineStr">
+        <is>
+          <t>Servo diagnostic boot synchronization</t>
+        </is>
+      </c>
+      <c r="E147" s="20" t="inlineStr">
+        <is>
+          <t>Bounded boot wait and partial-line drain before fresh identity/status; retain fatal runtime errors, no motion retries and prompt cancellation cleanup</t>
+        </is>
+      </c>
+      <c r="F147" s="20" t="inlineStr">
+        <is>
+          <t>firmware/three_board/README.md</t>
+        </is>
+      </c>
+      <c r="G147" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H147" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I147" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J147" s="20" t="inlineStr">
+        <is>
+          <t>31 simulated servo checks passed, including boot partial-line recovery, cancellation, persistent noise and fatal handshake/motion errors. Required gate passed: ======================= 48 passed, 4 warnings in 21.41s =======================; ================= 563 passed, 1 skipped in 331.44s (0:05:31) ==================. Dashboard build passed. Physical hardware untouched; actual cause of reported malformed serial input remains unverified.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(edge): resolve camera staleness false abort, port locking, and add batch finish button
</commit_message>
<xml_diff>
--- a/docs/OvaLens_Capstone_Feature_Checklist.xlsx
+++ b/docs/OvaLens_Capstone_Feature_Checklist.xlsx
@@ -871,7 +871,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:J147"/>
+  <dimension ref="A3:J148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8386,6 +8386,58 @@
         </is>
       </c>
     </row>
+    <row r="148">
+      <c r="A148" s="19" t="inlineStr">
+        <is>
+          <t>TASK-NEW-EDGE-LIGHT-TEST-01</t>
+        </is>
+      </c>
+      <c r="B148" s="19" t="inlineStr">
+        <is>
+          <t>Phase 4B: Edge CV</t>
+        </is>
+      </c>
+      <c r="C148" s="20" t="inlineStr">
+        <is>
+          <t>Edge / Firmware</t>
+        </is>
+      </c>
+      <c r="D148" s="20" t="inlineStr">
+        <is>
+          <t>Standalone COM9 light test</t>
+        </is>
+      </c>
+      <c r="E148" s="20" t="inlineStr">
+        <is>
+          <t>Bounded on/off test with identity/output confirmation, serial boot synchronization and off/stop cleanup</t>
+        </is>
+      </c>
+      <c r="F148" s="20" t="inlineStr">
+        <is>
+          <t>firmware/three_board/README.md</t>
+        </is>
+      </c>
+      <c r="G148" s="19" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="H148" s="21" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="I148" s="19" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="J148" s="20" t="inlineStr">
+        <is>
+          <t>Implementation and simulated verification pending; no physical hardware access.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>